<commit_message>
Replace overload relays with Siemens DIN-rail MPCBs
Co-authored-by: XDWOLLEN <74133863+XDWOLLEN@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/pano_varyasyon_maliyet.xlsx
+++ b/pano_varyasyon_maliyet.xlsx
@@ -142,7 +142,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
@@ -394,7 +394,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">LS MMS-32S motor koruma şalteri, 40 A sınıfı</t>
+          <t xml:space="preserve">Siemens SIRIUS 3RV2031-4UA10, 28–40 A motor koruma şalteri (vidalı bağlantı, DIN rayı)</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -402,19 +402,21 @@
           <t xml:space="preserve">Ürün sayfası</t>
         </is>
       </c>
-      <c r="C8" s="8">
-        <v>1237.42</v>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Teklif gerekli</t>
+        </is>
       </c>
       <c r="D8" s="5">
         <v>20</v>
       </c>
       <c r="E8" s="9">
-        <f>C8*D8</f>
+        <f>IF(ISNUMBER(C8),C8*D8,"Teklif gerekli")</f>
         <v/>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">LS MMS-32S motor koruma şalteri, 40 A sınıfı</t>
+          <t xml:space="preserve">Siemens SIRIUS 3RV2031-4UA10, 28–40 A motor koruma şalteri (vidalı bağlantı, DIN rayı)</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
@@ -422,19 +424,21 @@
           <t xml:space="preserve">Ürün sayfası</t>
         </is>
       </c>
-      <c r="I8" s="8">
-        <v>1237.42</v>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Teklif gerekli</t>
+        </is>
       </c>
       <c r="J8" s="5">
         <v>20</v>
       </c>
       <c r="K8" s="9">
-        <f>I8*J8</f>
+        <f>IF(ISNUMBER(I8),I8*J8,"Teklif gerekli")</f>
         <v/>
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">LS MMS-32S motor koruma şalteri, 40 A sınıfı</t>
+          <t xml:space="preserve">Siemens SIRIUS 3RV2031-4UA10, 28–40 A motor koruma şalteri (vidalı bağlantı, DIN rayı)</t>
         </is>
       </c>
       <c r="N8" s="6" t="inlineStr">
@@ -442,19 +446,21 @@
           <t xml:space="preserve">Ürün sayfası</t>
         </is>
       </c>
-      <c r="O8" s="8">
-        <v>1237.42</v>
+      <c r="O8" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Teklif gerekli</t>
+        </is>
       </c>
       <c r="P8" s="5">
         <v>20</v>
       </c>
       <c r="Q8" s="9">
-        <f>O8*P8</f>
+        <f>IF(ISNUMBER(O8),O8*P8,"Teklif gerekli")</f>
         <v/>
       </c>
       <c r="S8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">LS MMS-32S motor koruma şalteri, 40 A sınıfı</t>
+          <t xml:space="preserve">Siemens SIRIUS 3RV2031-4UA10, 28–40 A motor koruma şalteri (vidalı bağlantı, DIN rayı)</t>
         </is>
       </c>
       <c r="T8" s="6" t="inlineStr">
@@ -462,14 +468,16 @@
           <t xml:space="preserve">Ürün sayfası</t>
         </is>
       </c>
-      <c r="U8" s="8">
-        <v>1237.42</v>
+      <c r="U8" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Teklif gerekli</t>
+        </is>
       </c>
       <c r="V8" s="5">
         <v>20</v>
       </c>
       <c r="W8" s="9">
-        <f>U8*V8</f>
+        <f>IF(ISNUMBER(U8),U8*V8,"Teklif gerekli")</f>
         <v/>
       </c>
     </row>
@@ -596,46 +604,6 @@
         <f>I10*J10</f>
         <v/>
       </c>
-      <c r="M10" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LS MT-32, 40 A termik röle</t>
-        </is>
-      </c>
-      <c r="N10" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ürün sayfası</t>
-        </is>
-      </c>
-      <c r="O10" s="8">
-        <v>1104.36</v>
-      </c>
-      <c r="P10" s="5">
-        <v>20</v>
-      </c>
-      <c r="Q10" s="9">
-        <f>O10*P10</f>
-        <v/>
-      </c>
-      <c r="S10" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LS MT-32, 40 A termik röle</t>
-        </is>
-      </c>
-      <c r="T10" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ürün sayfası</t>
-        </is>
-      </c>
-      <c r="U10" s="8">
-        <v>1104.36</v>
-      </c>
-      <c r="V10" s="5">
-        <v>20</v>
-      </c>
-      <c r="W10" s="9">
-        <f>U10*V10</f>
-        <v/>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -1056,7 +1024,7 @@
         </is>
       </c>
       <c r="E17" s="11">
-        <f>SUM(E7:E16)</f>
+        <f>IF(COUNT(E7:E16)&lt;COUNTA(A7:A16),"TEKLİF GEREKLİ",SUM(E7:E16))</f>
         <v/>
       </c>
       <c r="G17" s="10" t="inlineStr">
@@ -1065,7 +1033,7 @@
         </is>
       </c>
       <c r="K17" s="11">
-        <f>SUM(K7:K16)</f>
+        <f>IF(COUNT(K7:K16)&lt;COUNTA(G7:G16),"TEKLİF GEREKLİ",SUM(K7:K16))</f>
         <v/>
       </c>
       <c r="M17" s="10" t="inlineStr">
@@ -1074,7 +1042,7 @@
         </is>
       </c>
       <c r="Q17" s="11">
-        <f>SUM(Q7:Q16)</f>
+        <f>IF(COUNT(Q7:Q16)&lt;COUNTA(M7:M16),"TEKLİF GEREKLİ",SUM(Q7:Q16))</f>
         <v/>
       </c>
       <c r="S17" s="10" t="inlineStr">
@@ -1083,7 +1051,7 @@
         </is>
       </c>
       <c r="W17" s="11">
-        <f>SUM(W7:W16)</f>
+        <f>IF(COUNT(W7:W16)&lt;COUNTA(S7:S16),"TEKLİF GEREKLİ",SUM(W7:W16))</f>
         <v/>
       </c>
     </row>
@@ -1200,7 +1168,7 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">LS MMS-32S motor koruma şalteri, 13 A sınıfı</t>
+          <t xml:space="preserve">Siemens SIRIUS 3RV2011-1KA10, 9–12,5 A motor koruma şalteri (vidalı bağlantı, DIN rayı)</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
@@ -1208,19 +1176,21 @@
           <t xml:space="preserve">Ürün sayfası</t>
         </is>
       </c>
-      <c r="C25" s="8">
-        <v>1237.42</v>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Teklif gerekli</t>
+        </is>
       </c>
       <c r="D25" s="5">
         <v>9</v>
       </c>
       <c r="E25" s="9">
-        <f>C25*D25</f>
+        <f>IF(ISNUMBER(C25),C25*D25,"Teklif gerekli")</f>
         <v/>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">LS MMS-32S motor koruma şalteri, 13 A sınıfı</t>
+          <t xml:space="preserve">Siemens SIRIUS 3RV2011-1KA10, 9–12,5 A motor koruma şalteri (vidalı bağlantı, DIN rayı)</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
@@ -1228,14 +1198,16 @@
           <t xml:space="preserve">Ürün sayfası</t>
         </is>
       </c>
-      <c r="I25" s="8">
-        <v>1237.42</v>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Teklif gerekli</t>
+        </is>
       </c>
       <c r="J25" s="5">
         <v>9</v>
       </c>
       <c r="K25" s="9">
-        <f>I25*J25</f>
+        <f>IF(ISNUMBER(I25),I25*J25,"Teklif gerekli")</f>
         <v/>
       </c>
     </row>
@@ -1281,48 +1253,7 @@
         <v/>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LS MT-32, 18 A termik röle</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ürün sayfası</t>
-        </is>
-      </c>
-      <c r="C27" s="8">
-        <v>1157.59</v>
-      </c>
-      <c r="D27" s="5">
-        <v>9</v>
-      </c>
-      <c r="E27" s="9">
-        <f>C27*D27</f>
-        <v/>
-      </c>
-      <c r="G27" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LS MT-32, 18 A termik röle</t>
-        </is>
-      </c>
-      <c r="H27" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ürün sayfası</t>
-        </is>
-      </c>
-      <c r="I27" s="8">
-        <v>1157.59</v>
-      </c>
-      <c r="J27" s="5">
-        <v>9</v>
-      </c>
-      <c r="K27" s="9">
-        <f>I27*J27</f>
-        <v/>
-      </c>
-    </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
@@ -1562,7 +1493,7 @@
         </is>
       </c>
       <c r="E34" s="11">
-        <f>SUM(E24:E33)</f>
+        <f>IF(COUNT(E24:E33)&lt;COUNTA(A24:A33),"TEKLİF GEREKLİ",SUM(E24:E33))</f>
         <v/>
       </c>
       <c r="G34" s="10" t="inlineStr">
@@ -1571,7 +1502,7 @@
         </is>
       </c>
       <c r="K34" s="11">
-        <f>SUM(K24:K33)</f>
+        <f>IF(COUNT(K24:K33)&lt;COUNTA(G24:G33),"TEKLİF GEREKLİ",SUM(K24:K33))</f>
         <v/>
       </c>
     </row>
@@ -1688,7 +1619,7 @@
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">LS MMS-32S motor koruma şalteri, 13 A sınıfı</t>
+          <t xml:space="preserve">Siemens SIRIUS 3RV2011-1KA10, 9–12,5 A motor koruma şalteri (vidalı bağlantı, DIN rayı)</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
@@ -1696,19 +1627,21 @@
           <t xml:space="preserve">Ürün sayfası</t>
         </is>
       </c>
-      <c r="C42" s="8">
-        <v>1237.42</v>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Teklif gerekli</t>
+        </is>
       </c>
       <c r="D42" s="5">
         <v>10</v>
       </c>
       <c r="E42" s="9">
-        <f>C42*D42</f>
+        <f>IF(ISNUMBER(C42),C42*D42,"Teklif gerekli")</f>
         <v/>
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">LS MMS-32S motor koruma şalteri, 13 A sınıfı</t>
+          <t xml:space="preserve">Siemens SIRIUS 3RV2011-1KA10, 9–12,5 A motor koruma şalteri (vidalı bağlantı, DIN rayı)</t>
         </is>
       </c>
       <c r="H42" s="6" t="inlineStr">
@@ -1716,14 +1649,16 @@
           <t xml:space="preserve">Ürün sayfası</t>
         </is>
       </c>
-      <c r="I42" s="8">
-        <v>1237.42</v>
+      <c r="I42" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Teklif gerekli</t>
+        </is>
       </c>
       <c r="J42" s="5">
         <v>10</v>
       </c>
       <c r="K42" s="9">
-        <f>I42*J42</f>
+        <f>IF(ISNUMBER(I42),I42*J42,"Teklif gerekli")</f>
         <v/>
       </c>
     </row>
@@ -1769,48 +1704,7 @@
         <v/>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LS MT-32, 18 A termik röle</t>
-        </is>
-      </c>
-      <c r="B44" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ürün sayfası</t>
-        </is>
-      </c>
-      <c r="C44" s="8">
-        <v>1157.59</v>
-      </c>
-      <c r="D44" s="5">
-        <v>10</v>
-      </c>
-      <c r="E44" s="9">
-        <f>C44*D44</f>
-        <v/>
-      </c>
-      <c r="G44" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LS MT-32, 18 A termik röle</t>
-        </is>
-      </c>
-      <c r="H44" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ürün sayfası</t>
-        </is>
-      </c>
-      <c r="I44" s="8">
-        <v>1157.59</v>
-      </c>
-      <c r="J44" s="5">
-        <v>10</v>
-      </c>
-      <c r="K44" s="9">
-        <f>I44*J44</f>
-        <v/>
-      </c>
-    </row>
+    <row r="44"/>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
@@ -2050,7 +1944,7 @@
         </is>
       </c>
       <c r="E51" s="11">
-        <f>SUM(E41:E50)</f>
+        <f>IF(COUNT(E41:E50)&lt;COUNTA(A41:A50),"TEKLİF GEREKLİ",SUM(E41:E50))</f>
         <v/>
       </c>
       <c r="G51" s="10" t="inlineStr">
@@ -2059,7 +1953,7 @@
         </is>
       </c>
       <c r="K51" s="11">
-        <f>SUM(K41:K50)</f>
+        <f>IF(COUNT(K41:K50)&lt;COUNTA(G41:G50),"TEKLİF GEREKLİ",SUM(K41:K50))</f>
         <v/>
       </c>
     </row>
@@ -2077,643 +1971,635 @@
     <mergeCell ref="G39:K39"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B7" ns1:id="rId1"/>
-    <hyperlink ref="B8" ns1:id="rId2"/>
-    <hyperlink ref="B9" ns1:id="rId3"/>
-    <hyperlink ref="B10" ns1:id="rId4"/>
-    <hyperlink ref="B11" ns1:id="rId5"/>
-    <hyperlink ref="B12" ns1:id="rId6"/>
-    <hyperlink ref="B13" ns1:id="rId7"/>
-    <hyperlink ref="H7" ns1:id="rId8"/>
-    <hyperlink ref="H8" ns1:id="rId9"/>
-    <hyperlink ref="H9" ns1:id="rId10"/>
-    <hyperlink ref="H10" ns1:id="rId11"/>
-    <hyperlink ref="H11" ns1:id="rId12"/>
-    <hyperlink ref="H12" ns1:id="rId13"/>
-    <hyperlink ref="N7" ns1:id="rId14"/>
-    <hyperlink ref="N8" ns1:id="rId15"/>
-    <hyperlink ref="N9" ns1:id="rId16"/>
-    <hyperlink ref="N10" ns1:id="rId17"/>
-    <hyperlink ref="N11" ns1:id="rId18"/>
-    <hyperlink ref="N12" ns1:id="rId19"/>
-    <hyperlink ref="N13" ns1:id="rId20"/>
-    <hyperlink ref="N14" ns1:id="rId21"/>
-    <hyperlink ref="T7" ns1:id="rId22"/>
-    <hyperlink ref="T8" ns1:id="rId23"/>
-    <hyperlink ref="T9" ns1:id="rId24"/>
-    <hyperlink ref="T10" ns1:id="rId25"/>
-    <hyperlink ref="T11" ns1:id="rId26"/>
-    <hyperlink ref="T12" ns1:id="rId27"/>
-    <hyperlink ref="T13" ns1:id="rId28"/>
-    <hyperlink ref="B24" ns1:id="rId29"/>
-    <hyperlink ref="B25" ns1:id="rId30"/>
-    <hyperlink ref="B26" ns1:id="rId31"/>
-    <hyperlink ref="B27" ns1:id="rId32"/>
-    <hyperlink ref="B28" ns1:id="rId33"/>
-    <hyperlink ref="B29" ns1:id="rId34"/>
-    <hyperlink ref="B30" ns1:id="rId35"/>
-    <hyperlink ref="B31" ns1:id="rId36"/>
-    <hyperlink ref="H24" ns1:id="rId37"/>
-    <hyperlink ref="H25" ns1:id="rId38"/>
-    <hyperlink ref="H26" ns1:id="rId39"/>
-    <hyperlink ref="H27" ns1:id="rId40"/>
-    <hyperlink ref="H28" ns1:id="rId41"/>
-    <hyperlink ref="H29" ns1:id="rId42"/>
-    <hyperlink ref="H30" ns1:id="rId43"/>
-    <hyperlink ref="B41" ns1:id="rId44"/>
-    <hyperlink ref="B42" ns1:id="rId45"/>
-    <hyperlink ref="B43" ns1:id="rId46"/>
-    <hyperlink ref="B44" ns1:id="rId47"/>
-    <hyperlink ref="B45" ns1:id="rId48"/>
-    <hyperlink ref="B46" ns1:id="rId49"/>
-    <hyperlink ref="B47" ns1:id="rId50"/>
-    <hyperlink ref="B48" ns1:id="rId51"/>
-    <hyperlink ref="H41" ns1:id="rId52"/>
-    <hyperlink ref="H42" ns1:id="rId53"/>
-    <hyperlink ref="H43" ns1:id="rId54"/>
-    <hyperlink ref="H44" ns1:id="rId55"/>
-    <hyperlink ref="H45" ns1:id="rId56"/>
-    <hyperlink ref="H46" ns1:id="rId57"/>
-    <hyperlink ref="H47" ns1:id="rId58"/>
-    <hyperlink ref="B15" ns1:id="rId59"/>
-    <hyperlink ref="B16" ns1:id="rId60"/>
-    <hyperlink ref="H15" ns1:id="rId61"/>
-    <hyperlink ref="H16" ns1:id="rId62"/>
-    <hyperlink ref="N15" ns1:id="rId63"/>
-    <hyperlink ref="N16" ns1:id="rId64"/>
-    <hyperlink ref="T15" ns1:id="rId65"/>
-    <hyperlink ref="T16" ns1:id="rId66"/>
-    <hyperlink ref="B32" ns1:id="rId67"/>
-    <hyperlink ref="B33" ns1:id="rId68"/>
-    <hyperlink ref="H32" ns1:id="rId69"/>
-    <hyperlink ref="H33" ns1:id="rId70"/>
-    <hyperlink ref="B49" ns1:id="rId71"/>
-    <hyperlink ref="B50" ns1:id="rId72"/>
-    <hyperlink ref="H49" ns1:id="rId73"/>
-    <hyperlink ref="H50" ns1:id="rId74"/>
+    <hyperlink ref="B7" r:id="rId1"/>
+    <hyperlink ref="B8" r:id="rId2"/>
+    <hyperlink ref="B9" r:id="rId3"/>
+    <hyperlink ref="B10" r:id="rId4"/>
+    <hyperlink ref="B11" r:id="rId5"/>
+    <hyperlink ref="B12" r:id="rId6"/>
+    <hyperlink ref="B13" r:id="rId7"/>
+    <hyperlink ref="H7" r:id="rId8"/>
+    <hyperlink ref="H8" r:id="rId9"/>
+    <hyperlink ref="H9" r:id="rId10"/>
+    <hyperlink ref="H10" r:id="rId11"/>
+    <hyperlink ref="H11" r:id="rId12"/>
+    <hyperlink ref="H12" r:id="rId13"/>
+    <hyperlink ref="N7" r:id="rId14"/>
+    <hyperlink ref="N8" r:id="rId15"/>
+    <hyperlink ref="N9" r:id="rId16"/>
+    <hyperlink ref="N11" r:id="rId18"/>
+    <hyperlink ref="N12" r:id="rId19"/>
+    <hyperlink ref="N13" r:id="rId20"/>
+    <hyperlink ref="N14" r:id="rId21"/>
+    <hyperlink ref="T7" r:id="rId22"/>
+    <hyperlink ref="T8" r:id="rId23"/>
+    <hyperlink ref="T9" r:id="rId24"/>
+    <hyperlink ref="T11" r:id="rId26"/>
+    <hyperlink ref="T12" r:id="rId27"/>
+    <hyperlink ref="T13" r:id="rId28"/>
+    <hyperlink ref="B24" r:id="rId29"/>
+    <hyperlink ref="B25" r:id="rId30"/>
+    <hyperlink ref="B26" r:id="rId31"/>
+    <hyperlink ref="B28" r:id="rId33"/>
+    <hyperlink ref="B29" r:id="rId34"/>
+    <hyperlink ref="B30" r:id="rId35"/>
+    <hyperlink ref="B31" r:id="rId36"/>
+    <hyperlink ref="H24" r:id="rId37"/>
+    <hyperlink ref="H25" r:id="rId38"/>
+    <hyperlink ref="H26" r:id="rId39"/>
+    <hyperlink ref="H28" r:id="rId41"/>
+    <hyperlink ref="H29" r:id="rId42"/>
+    <hyperlink ref="H30" r:id="rId43"/>
+    <hyperlink ref="B41" r:id="rId44"/>
+    <hyperlink ref="B42" r:id="rId45"/>
+    <hyperlink ref="B43" r:id="rId46"/>
+    <hyperlink ref="B45" r:id="rId48"/>
+    <hyperlink ref="B46" r:id="rId49"/>
+    <hyperlink ref="B47" r:id="rId50"/>
+    <hyperlink ref="B48" r:id="rId51"/>
+    <hyperlink ref="H41" r:id="rId52"/>
+    <hyperlink ref="H42" r:id="rId53"/>
+    <hyperlink ref="H43" r:id="rId54"/>
+    <hyperlink ref="H45" r:id="rId56"/>
+    <hyperlink ref="H46" r:id="rId57"/>
+    <hyperlink ref="H47" r:id="rId58"/>
+    <hyperlink ref="B15" r:id="rId59"/>
+    <hyperlink ref="B16" r:id="rId60"/>
+    <hyperlink ref="H15" r:id="rId61"/>
+    <hyperlink ref="H16" r:id="rId62"/>
+    <hyperlink ref="N15" r:id="rId63"/>
+    <hyperlink ref="N16" r:id="rId64"/>
+    <hyperlink ref="T15" r:id="rId65"/>
+    <hyperlink ref="T16" r:id="rId66"/>
+    <hyperlink ref="B32" r:id="rId67"/>
+    <hyperlink ref="B33" r:id="rId68"/>
+    <hyperlink ref="H32" r:id="rId69"/>
+    <hyperlink ref="H33" r:id="rId70"/>
+    <hyperlink ref="B49" r:id="rId71"/>
+    <hyperlink ref="B50" r:id="rId72"/>
+    <hyperlink ref="H49" r:id="rId73"/>
+    <hyperlink ref="H50" r:id="rId74"/>
   </hyperlinks>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <cols>
-    <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="23" customWidth="1"/>
-    <col min="3" max="3" width="31" customWidth="1"/>
-    <col min="4" max="4" width="88" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">VARSAYIMLAR, SINIRLAR VE FİYAT KAYNAKLARI</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Çalışma tarihi</t>
-        </is>
-      </c>
-      <c r="B3" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">08.10.2026; arama sonuçlarında görülen çevrimiçi liste fiyatları kullanılmıştır.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Adet varsayımları</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pano 1: 14 + 6 = 20 adet 18,5 kW pompa. Pano 2: 4 + 5 = 9 adet 5,5 kW pompa. Pano 3: 7 + 3 = 10 adet 5,5 kW fan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yol verme</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sürücüsüz varyasyonlar yıldız-üçgen kabul edilmiştir: motor başına 3 kontaktör, motor koruma/termik ve (varsa) 1 zaman rölesi.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">VFD + zaman rölesi</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bu tabloda zaman rölesi yıldız-üçgen için değil, VFD motorlarının kademeli devreye alınması için ek bütçe kalemidir; sürücünün dahili hızlanma rampası vardır.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Zaman rölesi</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ENDA ATSP4 bağlantısı genel amaçlı analog zaman rölesi ürün sayfasıdır. Yıldız-üçgen işlev/çıkış kontak düzeni ve bobin gerilimi proje öncesi üretici dokümanından doğrulanmalıdır.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Kontrol/IO</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Waveshare 8DI/8DO kartı kullanıcı varsayımıyla mevcut kabul edilmiş ve maliyeti 0 TL yazılmıştır. 16 kanallı Modbus röle kartları 16 çıkış/motor kontaktör bobinleri varsayımıyla sayılmıştır.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Eksik kontrol kalemi</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gerekli dijital giriş sayısı 8DI kapasitesini aşar; dijital giriş genişletmesi, haberleşme konfigürasyonu ve güvenli fail-safe tasarım maliyeti bu dosyada fiyatlandırılmamıştır.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yıldız-üçgen emniyeti</t>
-        </is>
-      </c>
-      <c r="B10" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ESP32 zamanlaması tek başına emniyet değildir; yıldız/üçgen kontaktörlerinde mekanik kilitleme ve karşılıklı NC elektriksel kilitleme ile donanımsal acil-stop/termik zinciri gerekir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Kapsam dışı</t>
-        </is>
-      </c>
-      <c r="B11" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pano kabini, bara, kablolama, klemens, fan/filtre, SPD, ana kumanda/koruma aksesuarları, saha mühendisliği, montaj, devreye alma, nakliye ve işçilik toplamda yoktur. Liste tam satın alma BOM’u/uygulama projesi değildir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Teknik onay</t>
-        </is>
-      </c>
-      <c r="B12" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Motor etiket akımı, kısa devre seviyesi, koordinasyon, kontaktör/termik ayarları, sürücü giriş koruması, ana şalter seçimi ve pano ısıl hesabı yetkili elektrik mühendisi tarafından doğrulanmalıdır.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fiyat/KDV</t>
-        </is>
-      </c>
-      <c r="B13" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Birim maliyetler TRY cinsindedir. Waveshare kart fiyatları kullanıcı tarafından belirtilmiştir (ESP32-S3 kartı 4.000 TL/adet; 16 kanal röle kartı 6.400 TL/adet). Diğer fiyatların KDV/iskonto durumu satıcıya göre değişir; toplamlar ön bütçedir, teklif değildir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Stok</t>
-        </is>
-      </c>
-      <c r="B14" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ürün bağlantıları satıcı/üretici ürün sayfalarına gider. Bu oturumda her satıcının sepetindeki canlı stok miktarı kesin olarak doğrulanamadı; sipariş öncesi stok, teslim süresi, güncel fiyat ve teknik model teyidi gerekir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bara boyutlandırma</t>
-        </is>
-      </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ön BOM varsayımı: 18,5 kW pano için 30×10 mm paralel faz baraları; 5,5 kW panolar için 20×5 mm faz baraları ve PE barası. Kesit/paralel sayısı, bara mesafesi, destek/izolasyon, sıcaklık artışı, kısa devre dayanımı ve IEC 61439 uygunluğu yetkili elektrik mühendisi tarafından hesaplanıp doğrulanmalıdır; bu satırlar kesin proje/uygulama onayı değildir. Fiyatlar yaklaşık ve KDV/işleme/kargo durumu teyit edilmelidir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Kalem</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Satıcı sayfası</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fiyata esas alınan tutar</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">18,5 kW Delta sürücü</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ürün sayfası</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">45.441,00 TL/adet</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sayhan çevrimiçi fiyatı; stok kontrolü gerekli.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1000 A kompakt şalter</t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ürün sayfası</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">121.951,64 TL/adet</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tümpa liste fiyatı.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">160 A kompakt şalter</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ürün sayfası</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4.530,79 TL/adet</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tümpa fiyatı + KDV olarak raporlandı.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">40 A motor koruma şalteri</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ürün sayfası</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.237,42 TL/adet</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sayhan indirimli fiyat; varyant/ayar aralığı teyidi.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">13 A motor koruma şalteri</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ürün sayfası</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.237,42 TL/adet</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sayhan indirimli fiyat; ayar aralığı 9–13 A.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">40 A / 18,5 kW kontaktör</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ürün sayfası</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5.170,00 TL/adet</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tümpa Siemens 24 V DC bobinli model.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Siemens 3RT2017-1BB41, 12 A / 5,5 kW kontaktör</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ürün sayfası</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.137,00 TL/adet + KDV</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Elpimshop ürün sayfası; stokta 10+ adet bilgisi arama anında listelenmiş. Bobin 24 V DC, 1NA; stok ve fiyatı sipariş öncesi teyit edin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">40 A termik röle</t>
-        </is>
-      </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ürün sayfası</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.104,36 TL/adet</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sayhan liste fiyatı; motor akımına göre ayar teyidi.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">18 A termik röle</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ürün sayfası</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.157,59 TL/adet</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sayhan liste fiyatı.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Analog zaman rölesi</t>
-        </is>
-      </c>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ürün sayfası</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.039,50 TL/adet</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sayhan indirimli fiyat.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">24 V / 10 A güç kaynağı</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ürün sayfası</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2.062,84 TL/adet</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huzur Elektromarket fiyatı + KDV olarak raporlandı.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Waveshare 16 kanallı Modbus Ethernet röle kartı</t>
-        </is>
-      </c>
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ürün sayfası</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6.400,00 TL/adet (kullanıcı tarafından belirtilen)</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Kullanıcı tarafından verilen birim fiyat; Waveshare ürün sayfasından model/tedarik uygunluğu teyit edin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Waveshare ESP32-S3-POE-ETH-8DI-8DO</t>
-        </is>
-      </c>
-      <c r="B29" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ürün sayfası</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4.000,00 TL/adet (kullanıcı tarafından belirtilen)</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Kullanıcı tarafından verilen birim fiyat; Waveshare ürün sayfasından model/tedarik uygunluğu teyit edin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bakır bara 30×10 mm × 3 m</t>
-        </is>
-      </c>
-      <c r="B31" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ürün sayfası</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">≈ 5.900 TL/bar</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Hepsiburada listelemesi; arama anında yaklaşık ürün fiyatı. Liste seçeneği ve uzunluk/fiyatı sipariş öncesi teyit edin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bakır bara 20×5 mm × 1 m</t>
-        </is>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ürün sayfası</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">≈ 1.800 TL/bar</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Hepsiburada ürün listesi; boy ve güncel fiyatı satın almadan önce teyit edin.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="14">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B15:D15"/>
-  </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="B17" ns1:id="rId1"/>
-    <hyperlink ref="B18" ns1:id="rId2"/>
-    <hyperlink ref="B19" ns1:id="rId3"/>
-    <hyperlink ref="B20" ns1:id="rId4"/>
-    <hyperlink ref="B21" ns1:id="rId5"/>
-    <hyperlink ref="B22" ns1:id="rId6"/>
-    <hyperlink ref="B23" ns1:id="rId7"/>
-    <hyperlink ref="B24" ns1:id="rId8"/>
-    <hyperlink ref="B25" ns1:id="rId9"/>
-    <hyperlink ref="B26" ns1:id="rId10"/>
-    <hyperlink ref="B27" ns1:id="rId11"/>
-    <hyperlink ref="B28" ns1:id="rId12"/>
-    <hyperlink ref="B29" ns1:id="rId13"/>
-    <hyperlink ref="B31" ns1:id="rId14"/>
-    <hyperlink ref="B32" ns1:id="rId15"/>
-  </hyperlinks>
-  <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
-</worksheet>
+<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <ns0:cols>
+    <ns0:col min="1" max="1" width="28" customWidth="1"/>
+    <ns0:col min="2" max="2" width="23" customWidth="1"/>
+    <ns0:col min="3" max="3" width="31" customWidth="1"/>
+    <ns0:col min="4" max="4" width="88" customWidth="1"/>
+  </ns0:cols>
+  <ns0:sheetData>
+    <ns0:row r="1">
+      <ns0:c r="A1" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">VARSAYIMLAR, SINIRLAR VE FİYAT KAYNAKLARI</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="3">
+      <ns0:c r="A3" s="3" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Çalışma tarihi</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B3" s="12" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">08.10.2026; arama sonuçlarında görülen çevrimiçi liste fiyatları kullanılmıştır.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="4">
+      <ns0:c r="A4" s="3" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Adet varsayımları</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B4" s="12" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Pano 1: 14 + 6 = 20 adet 18,5 kW pompa. Pano 2: 4 + 5 = 9 adet 5,5 kW pompa. Pano 3: 7 + 3 = 10 adet 5,5 kW fan.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="5">
+      <ns0:c r="A5" s="3" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Motor koruması</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B5" s="12" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Motor başına tek Siemens 3RV2 motor koruma şalteri kullanılır; ayrı termik röle satırları kaldırılmıştır. Sürücüsüz Y/Δ devrelerinde motor akım ayarı ve koordinasyon mühendislik hesabıyla doğrulanmalıdır.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="6">
+      <ns0:c r="A6" s="3" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">VFD + zaman rölesi</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B6" s="12" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Bu tabloda zaman rölesi yıldız-üçgen için değil, VFD motorlarının kademeli devreye alınması için ek bütçe kalemidir; sürücünün dahili hızlanma rampası vardır.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="7">
+      <ns0:c r="A7" s="3" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Zaman rölesi</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B7" s="12" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">ENDA ATSP4 bağlantısı genel amaçlı analog zaman rölesi ürün sayfasıdır. Yıldız-üçgen işlev/çıkış kontak düzeni ve bobin gerilimi proje öncesi üretici dokümanından doğrulanmalıdır.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="8">
+      <ns0:c r="A8" s="3" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Kontrol/IO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B8" s="12" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Waveshare 8DI/8DO kartı kullanıcı varsayımıyla mevcut kabul edilmiş ve maliyeti 0 TL yazılmıştır. 16 kanallı Modbus röle kartları 16 çıkış/motor kontaktör bobinleri varsayımıyla sayılmıştır.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="9">
+      <ns0:c r="A9" s="3" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Eksik kontrol kalemi</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B9" s="12" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Gerekli dijital giriş sayısı 8DI kapasitesini aşar; dijital giriş genişletmesi, haberleşme konfigürasyonu ve güvenli fail-safe tasarım maliyeti bu dosyada fiyatlandırılmamıştır.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="10">
+      <ns0:c r="A10" s="3" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Yıldız-üçgen emniyeti</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B10" s="12" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">ESP32 zamanlaması tek başına emniyet değildir; yıldız/üçgen kontaktörlerinde mekanik kilitleme ve karşılıklı NC elektriksel kilitleme ile donanımsal acil-stop ve uygun motor koruma şalteri zinciri gerekir.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="11">
+      <ns0:c r="A11" s="3" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Kapsam dışı</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B11" s="12" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Pano kabini, bara, kablolama, klemens, fan/filtre, SPD, ana kumanda/koruma aksesuarları, saha mühendisliği, montaj, devreye alma, nakliye ve işçilik toplamda yoktur. Liste tam satın alma BOM’u/uygulama projesi değildir.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="12">
+      <ns0:c r="A12" s="3" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Teknik onay</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B12" s="12" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Motor etiket akımı, kısa devre seviyesi, koordinasyon, Siemens motor koruma şalteri ayar aralığı, sürücü giriş koruması, ana şalter seçimi ve pano ısıl hesabı yetkili elektrik mühendisi tarafından doğrulanmalıdır.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="13">
+      <ns0:c r="A13" s="3" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Fiyat/KDV</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B13" s="12" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Birim maliyetler TRY cinsindedir. Waveshare kart fiyatları kullanıcı tarafından belirtilmiştir (ESP32-S3 kartı 4.000 TL/adet; 16 kanal röle kartı 6.400 TL/adet). Diğer fiyatların KDV/iskonto durumu satıcıya göre değişir; toplamlar ön bütçedir, teklif değildir.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="14">
+      <ns0:c r="A14" s="3" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Stok / fiyat</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B14" s="12" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">MPCB bağlantıları Siemens ürün kataloğuna gider; Türkiye satıcılarından fiyat/teslimat teklifi alınmalıdır. Güncel satıcı stoku ve KDV dahil fiyat teyit edilmediğinden motor koruma şalteri fiyatları ve pano toplamları “Teklif gerekli” görünür.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="15">
+      <ns0:c r="A15" s="3" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Bara boyutlandırma</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B15" s="12" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Ön BOM varsayımı: 18,5 kW pano için 30×10 mm paralel faz baraları; 5,5 kW panolar için 20×5 mm faz baraları ve PE barası. Kesit/paralel sayısı, bara mesafesi, destek/izolasyon, sıcaklık artışı, kısa devre dayanımı ve IEC 61439 uygunluğu yetkili elektrik mühendisi tarafından hesaplanıp doğrulanmalıdır; bu satırlar kesin proje/uygulama onayı değildir. Fiyatlar yaklaşık ve KDV/işleme/kargo durumu teyit edilmelidir.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="16">
+      <ns0:c r="A16" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Kalem</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B16" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Satıcı sayfası</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C16" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Fiyata esas alınan tutar</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D16" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Not</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="17">
+      <ns0:c r="A17" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">18,5 kW Delta sürücü</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B17" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C17" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">45.441,00 TL/adet</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D17" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Sayhan çevrimiçi fiyatı; stok kontrolü gerekli.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="18">
+      <ns0:c r="A18" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">1000 A kompakt şalter</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B18" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C18" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">121.951,64 TL/adet</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D18" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Tümpa liste fiyatı.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="19">
+      <ns0:c r="A19" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">160 A kompakt şalter</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B19" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C19" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">4.530,79 TL/adet</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D19" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Tümpa fiyatı + KDV olarak raporlandı.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="20">
+      <ns0:c r="A20" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">18,5 kW motor koruma şalteri</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B20" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C20" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Teklif gerekli</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D20" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Siemens 3RV2031-4UA10, 28–40 A; 3RV2 S2, vidalı bağlantı, raya montaj. Üretici kataloğu; fiyat için Türkiye satıcı teklifi gerekli.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="21">
+      <ns0:c r="A21" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">5,5 kW motor koruma şalteri</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B21" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C21" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Teklif gerekli</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D21" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Siemens 3RV2011-1KA10, 9–12,5 A; 3RV2 S00, vidalı bağlantı, raya montaj. Üretici kataloğu; fiyat için Türkiye satıcı teklifi gerekli.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="22">
+      <ns0:c r="A22" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">40 A / 18,5 kW kontaktör</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B22" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C22" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">5.170,00 TL/adet</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D22" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Tümpa Siemens 24 V DC bobinli model.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="23">
+      <ns0:c r="A23" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Siemens 3RT2017-1BB41, 12 A / 5,5 kW kontaktör</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B23" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C23" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">1.137,00 TL/adet + KDV</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D23" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Elpimshop ürün sayfası; stokta 10+ adet bilgisi arama anında listelenmiş. Bobin 24 V DC, 1NA; stok ve fiyatı sipariş öncesi teyit edin.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="24">
+      <ns0:c r="A24" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Eski 40 A termik röle</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B24" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Kullanılmıyor; ilgili termik röle satırları Siemens motor koruma şalteriyle tek cihazda birleştirildi.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C24" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">—</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D24" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Ayrı termik röle kullanılmıyor.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="25">
+      <ns0:c r="A25" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Eski 18 A termik röle</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B25" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Kullanılmıyor; ilgili termik röle satırları Siemens motor koruma şalteriyle tek cihazda birleştirildi.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C25" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">—</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D25" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Ayrı termik röle kullanılmıyor.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="26">
+      <ns0:c r="A26" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Analog zaman rölesi</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B26" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C26" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">1.039,50 TL/adet</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D26" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Sayhan indirimli fiyat.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="27">
+      <ns0:c r="A27" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">24 V / 10 A güç kaynağı</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B27" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C27" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2.062,84 TL/adet</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D27" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Huzur Elektromarket fiyatı + KDV olarak raporlandı.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="28">
+      <ns0:c r="A28" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Waveshare 16 kanallı Modbus Ethernet röle kartı</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B28" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C28" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">6.400,00 TL/adet (kullanıcı tarafından belirtilen)</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D28" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Kullanıcı tarafından verilen birim fiyat; Waveshare ürün sayfasından model/tedarik uygunluğu teyit edin.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="29">
+      <ns0:c r="A29" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Waveshare ESP32-S3-POE-ETH-8DI-8DO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B29" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C29" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">4.000,00 TL/adet (kullanıcı tarafından belirtilen)</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D29" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Kullanıcı tarafından verilen birim fiyat; Waveshare ürün sayfasından model/tedarik uygunluğu teyit edin.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="31">
+      <ns0:c r="A31" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Bakır bara 30×10 mm × 3 m</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B31" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C31" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">≈ 5.900 TL/bar</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D31" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Hepsiburada listelemesi; arama anında yaklaşık ürün fiyatı. Liste seçeneği ve uzunluk/fiyatı sipariş öncesi teyit edin.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="32">
+      <ns0:c r="A32" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Bakır bara 20×5 mm × 1 m</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B32" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C32" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">≈ 1.800 TL/bar</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D32" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Hepsiburada ürün listesi; boy ve güncel fiyatı satın almadan önce teyit edin.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+  </ns0:sheetData>
+  <ns0:mergeCells count="14">
+    <ns0:mergeCell ref="A1:D1"/>
+    <ns0:mergeCell ref="B3:D3"/>
+    <ns0:mergeCell ref="B4:D4"/>
+    <ns0:mergeCell ref="B5:D5"/>
+    <ns0:mergeCell ref="B6:D6"/>
+    <ns0:mergeCell ref="B7:D7"/>
+    <ns0:mergeCell ref="B8:D8"/>
+    <ns0:mergeCell ref="B9:D9"/>
+    <ns0:mergeCell ref="B10:D10"/>
+    <ns0:mergeCell ref="B11:D11"/>
+    <ns0:mergeCell ref="B12:D12"/>
+    <ns0:mergeCell ref="B13:D13"/>
+    <ns0:mergeCell ref="B14:D14"/>
+    <ns0:mergeCell ref="B15:D15"/>
+  </ns0:mergeCells>
+  <ns0:hyperlinks>
+    <ns0:hyperlink ref="B17" r:id="rId1"/>
+    <ns0:hyperlink ref="B18" r:id="rId2"/>
+    <ns0:hyperlink ref="B19" r:id="rId3"/>
+    <ns0:hyperlink ref="B20" r:id="rId4"/>
+    <ns0:hyperlink ref="B21" r:id="rId5"/>
+    <ns0:hyperlink ref="B22" r:id="rId6"/>
+    <ns0:hyperlink ref="B23" r:id="rId7"/>
+    <ns0:hyperlink ref="B26" r:id="rId10"/>
+    <ns0:hyperlink ref="B27" r:id="rId11"/>
+    <ns0:hyperlink ref="B28" r:id="rId12"/>
+    <ns0:hyperlink ref="B29" r:id="rId13"/>
+    <ns0:hyperlink ref="B31" r:id="rId14"/>
+    <ns0:hyperlink ref="B32" r:id="rId15"/>
+  </ns0:hyperlinks>
+  <ns0:pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+</ns0:worksheet>
 </file>
</xml_diff>

<commit_message>
Use supplied Elektrix Siemens 40A breaker
Co-authored-by: XDWOLLEN <74133863+XDWOLLEN@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/pano_varyasyon_maliyet.xlsx
+++ b/pano_varyasyon_maliyet.xlsx
@@ -394,7 +394,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Siemens SIRIUS 3RV2031-4UA10, 28–40 A motor koruma şalteri (vidalı bağlantı, DIN rayı)</t>
+          <t xml:space="preserve">Siemens SIRIUS 3RV2021-4FA10, 34–40 A motor koruma şalteri (vidalı bağlantı, DIN rayı)</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -402,10 +402,8 @@
           <t xml:space="preserve">Ürün sayfası</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Teklif gerekli</t>
-        </is>
+      <c r="C8" s="8">
+        <v>5946.48</v>
       </c>
       <c r="D8" s="5">
         <v>20</v>
@@ -416,7 +414,7 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Siemens SIRIUS 3RV2031-4UA10, 28–40 A motor koruma şalteri (vidalı bağlantı, DIN rayı)</t>
+          <t xml:space="preserve">Siemens SIRIUS 3RV2021-4FA10, 34–40 A motor koruma şalteri (vidalı bağlantı, DIN rayı)</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
@@ -424,10 +422,8 @@
           <t xml:space="preserve">Ürün sayfası</t>
         </is>
       </c>
-      <c r="I8" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Teklif gerekli</t>
-        </is>
+      <c r="I8" s="8">
+        <v>5946.48</v>
       </c>
       <c r="J8" s="5">
         <v>20</v>
@@ -438,7 +434,7 @@
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Siemens SIRIUS 3RV2031-4UA10, 28–40 A motor koruma şalteri (vidalı bağlantı, DIN rayı)</t>
+          <t xml:space="preserve">Siemens SIRIUS 3RV2021-4FA10, 34–40 A motor koruma şalteri (vidalı bağlantı, DIN rayı)</t>
         </is>
       </c>
       <c r="N8" s="6" t="inlineStr">
@@ -446,10 +442,8 @@
           <t xml:space="preserve">Ürün sayfası</t>
         </is>
       </c>
-      <c r="O8" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Teklif gerekli</t>
-        </is>
+      <c r="O8" s="8">
+        <v>5946.48</v>
       </c>
       <c r="P8" s="5">
         <v>20</v>
@@ -460,7 +454,7 @@
       </c>
       <c r="S8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Siemens SIRIUS 3RV2031-4UA10, 28–40 A motor koruma şalteri (vidalı bağlantı, DIN rayı)</t>
+          <t xml:space="preserve">Siemens SIRIUS 3RV2021-4FA10, 34–40 A motor koruma şalteri (vidalı bağlantı, DIN rayı)</t>
         </is>
       </c>
       <c r="T8" s="6" t="inlineStr">
@@ -468,10 +462,8 @@
           <t xml:space="preserve">Ürün sayfası</t>
         </is>
       </c>
-      <c r="U8" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Teklif gerekli</t>
-        </is>
+      <c r="U8" s="8">
+        <v>5946.48</v>
       </c>
       <c r="V8" s="5">
         <v>20</v>
@@ -2045,561 +2037,561 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <ns0:cols>
-    <ns0:col min="1" max="1" width="28" customWidth="1"/>
-    <ns0:col min="2" max="2" width="23" customWidth="1"/>
-    <ns0:col min="3" max="3" width="31" customWidth="1"/>
-    <ns0:col min="4" max="4" width="88" customWidth="1"/>
-  </ns0:cols>
-  <ns0:sheetData>
-    <ns0:row r="1">
-      <ns0:c r="A1" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">VARSAYIMLAR, SINIRLAR VE FİYAT KAYNAKLARI</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="3">
-      <ns0:c r="A3" s="3" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Çalışma tarihi</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B3" s="12" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">08.10.2026; arama sonuçlarında görülen çevrimiçi liste fiyatları kullanılmıştır.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="4">
-      <ns0:c r="A4" s="3" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Adet varsayımları</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B4" s="12" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Pano 1: 14 + 6 = 20 adet 18,5 kW pompa. Pano 2: 4 + 5 = 9 adet 5,5 kW pompa. Pano 3: 7 + 3 = 10 adet 5,5 kW fan.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="5">
-      <ns0:c r="A5" s="3" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Motor koruması</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B5" s="12" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Motor başına tek Siemens 3RV2 motor koruma şalteri kullanılır; ayrı termik röle satırları kaldırılmıştır. Sürücüsüz Y/Δ devrelerinde motor akım ayarı ve koordinasyon mühendislik hesabıyla doğrulanmalıdır.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="6">
-      <ns0:c r="A6" s="3" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">VFD + zaman rölesi</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B6" s="12" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Bu tabloda zaman rölesi yıldız-üçgen için değil, VFD motorlarının kademeli devreye alınması için ek bütçe kalemidir; sürücünün dahili hızlanma rampası vardır.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="7">
-      <ns0:c r="A7" s="3" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Zaman rölesi</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B7" s="12" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">ENDA ATSP4 bağlantısı genel amaçlı analog zaman rölesi ürün sayfasıdır. Yıldız-üçgen işlev/çıkış kontak düzeni ve bobin gerilimi proje öncesi üretici dokümanından doğrulanmalıdır.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="8">
-      <ns0:c r="A8" s="3" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Kontrol/IO</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B8" s="12" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Waveshare 8DI/8DO kartı kullanıcı varsayımıyla mevcut kabul edilmiş ve maliyeti 0 TL yazılmıştır. 16 kanallı Modbus röle kartları 16 çıkış/motor kontaktör bobinleri varsayımıyla sayılmıştır.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="9">
-      <ns0:c r="A9" s="3" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Eksik kontrol kalemi</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B9" s="12" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Gerekli dijital giriş sayısı 8DI kapasitesini aşar; dijital giriş genişletmesi, haberleşme konfigürasyonu ve güvenli fail-safe tasarım maliyeti bu dosyada fiyatlandırılmamıştır.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="10">
-      <ns0:c r="A10" s="3" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Yıldız-üçgen emniyeti</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B10" s="12" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">ESP32 zamanlaması tek başına emniyet değildir; yıldız/üçgen kontaktörlerinde mekanik kilitleme ve karşılıklı NC elektriksel kilitleme ile donanımsal acil-stop ve uygun motor koruma şalteri zinciri gerekir.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="11">
-      <ns0:c r="A11" s="3" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Kapsam dışı</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B11" s="12" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Pano kabini, bara, kablolama, klemens, fan/filtre, SPD, ana kumanda/koruma aksesuarları, saha mühendisliği, montaj, devreye alma, nakliye ve işçilik toplamda yoktur. Liste tam satın alma BOM’u/uygulama projesi değildir.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="12">
-      <ns0:c r="A12" s="3" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Teknik onay</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B12" s="12" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Motor etiket akımı, kısa devre seviyesi, koordinasyon, Siemens motor koruma şalteri ayar aralığı, sürücü giriş koruması, ana şalter seçimi ve pano ısıl hesabı yetkili elektrik mühendisi tarafından doğrulanmalıdır.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="13">
-      <ns0:c r="A13" s="3" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Fiyat/KDV</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B13" s="12" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Birim maliyetler TRY cinsindedir. Waveshare kart fiyatları kullanıcı tarafından belirtilmiştir (ESP32-S3 kartı 4.000 TL/adet; 16 kanal röle kartı 6.400 TL/adet). Diğer fiyatların KDV/iskonto durumu satıcıya göre değişir; toplamlar ön bütçedir, teklif değildir.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="14">
-      <ns0:c r="A14" s="3" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Stok / fiyat</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B14" s="12" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">MPCB bağlantıları Siemens ürün kataloğuna gider; Türkiye satıcılarından fiyat/teslimat teklifi alınmalıdır. Güncel satıcı stoku ve KDV dahil fiyat teyit edilmediğinden motor koruma şalteri fiyatları ve pano toplamları “Teklif gerekli” görünür.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="15">
-      <ns0:c r="A15" s="3" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Bara boyutlandırma</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B15" s="12" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Ön BOM varsayımı: 18,5 kW pano için 30×10 mm paralel faz baraları; 5,5 kW panolar için 20×5 mm faz baraları ve PE barası. Kesit/paralel sayısı, bara mesafesi, destek/izolasyon, sıcaklık artışı, kısa devre dayanımı ve IEC 61439 uygunluğu yetkili elektrik mühendisi tarafından hesaplanıp doğrulanmalıdır; bu satırlar kesin proje/uygulama onayı değildir. Fiyatlar yaklaşık ve KDV/işleme/kargo durumu teyit edilmelidir.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="16">
-      <ns0:c r="A16" s="4" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Kalem</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B16" s="4" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Satıcı sayfası</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C16" s="4" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Fiyata esas alınan tutar</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D16" s="4" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Not</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="17">
-      <ns0:c r="A17" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">18,5 kW Delta sürücü</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B17" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C17" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">45.441,00 TL/adet</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D17" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Sayhan çevrimiçi fiyatı; stok kontrolü gerekli.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="18">
-      <ns0:c r="A18" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">1000 A kompakt şalter</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B18" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C18" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">121.951,64 TL/adet</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D18" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Tümpa liste fiyatı.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="19">
-      <ns0:c r="A19" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">160 A kompakt şalter</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B19" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C19" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">4.530,79 TL/adet</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D19" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Tümpa fiyatı + KDV olarak raporlandı.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="20">
-      <ns0:c r="A20" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">18,5 kW motor koruma şalteri</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B20" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C20" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Teklif gerekli</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D20" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Siemens 3RV2031-4UA10, 28–40 A; 3RV2 S2, vidalı bağlantı, raya montaj. Üretici kataloğu; fiyat için Türkiye satıcı teklifi gerekli.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="21">
-      <ns0:c r="A21" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">5,5 kW motor koruma şalteri</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B21" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C21" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Teklif gerekli</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D21" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Siemens 3RV2011-1KA10, 9–12,5 A; 3RV2 S00, vidalı bağlantı, raya montaj. Üretici kataloğu; fiyat için Türkiye satıcı teklifi gerekli.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="22">
-      <ns0:c r="A22" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">40 A / 18,5 kW kontaktör</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B22" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C22" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">5.170,00 TL/adet</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D22" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Tümpa Siemens 24 V DC bobinli model.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="23">
-      <ns0:c r="A23" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Siemens 3RT2017-1BB41, 12 A / 5,5 kW kontaktör</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B23" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C23" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">1.137,00 TL/adet + KDV</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D23" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Elpimshop ürün sayfası; stokta 10+ adet bilgisi arama anında listelenmiş. Bobin 24 V DC, 1NA; stok ve fiyatı sipariş öncesi teyit edin.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="24">
-      <ns0:c r="A24" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Eski 40 A termik röle</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B24" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Kullanılmıyor; ilgili termik röle satırları Siemens motor koruma şalteriyle tek cihazda birleştirildi.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C24" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">—</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D24" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Ayrı termik röle kullanılmıyor.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="25">
-      <ns0:c r="A25" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Eski 18 A termik röle</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B25" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Kullanılmıyor; ilgili termik röle satırları Siemens motor koruma şalteriyle tek cihazda birleştirildi.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C25" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">—</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D25" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Ayrı termik röle kullanılmıyor.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="26">
-      <ns0:c r="A26" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Analog zaman rölesi</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B26" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C26" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">1.039,50 TL/adet</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D26" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Sayhan indirimli fiyat.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="27">
-      <ns0:c r="A27" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">24 V / 10 A güç kaynağı</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B27" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C27" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2.062,84 TL/adet</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D27" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Huzur Elektromarket fiyatı + KDV olarak raporlandı.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="28">
-      <ns0:c r="A28" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Waveshare 16 kanallı Modbus Ethernet röle kartı</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B28" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C28" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">6.400,00 TL/adet (kullanıcı tarafından belirtilen)</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D28" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Kullanıcı tarafından verilen birim fiyat; Waveshare ürün sayfasından model/tedarik uygunluğu teyit edin.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="29">
-      <ns0:c r="A29" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Waveshare ESP32-S3-POE-ETH-8DI-8DO</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B29" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C29" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">4.000,00 TL/adet (kullanıcı tarafından belirtilen)</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D29" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Kullanıcı tarafından verilen birim fiyat; Waveshare ürün sayfasından model/tedarik uygunluğu teyit edin.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="31">
-      <ns0:c r="A31" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Bakır bara 30×10 mm × 3 m</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B31" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C31" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">≈ 5.900 TL/bar</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D31" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Hepsiburada listelemesi; arama anında yaklaşık ürün fiyatı. Liste seçeneği ve uzunluk/fiyatı sipariş öncesi teyit edin.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="32">
-      <ns0:c r="A32" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Bakır bara 20×5 mm × 1 m</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B32" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C32" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">≈ 1.800 TL/bar</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D32" s="5" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Hepsiburada ürün listesi; boy ve güncel fiyatı satın almadan önce teyit edin.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-  </ns0:sheetData>
-  <ns0:mergeCells count="14">
-    <ns0:mergeCell ref="A1:D1"/>
-    <ns0:mergeCell ref="B3:D3"/>
-    <ns0:mergeCell ref="B4:D4"/>
-    <ns0:mergeCell ref="B5:D5"/>
-    <ns0:mergeCell ref="B6:D6"/>
-    <ns0:mergeCell ref="B7:D7"/>
-    <ns0:mergeCell ref="B8:D8"/>
-    <ns0:mergeCell ref="B9:D9"/>
-    <ns0:mergeCell ref="B10:D10"/>
-    <ns0:mergeCell ref="B11:D11"/>
-    <ns0:mergeCell ref="B12:D12"/>
-    <ns0:mergeCell ref="B13:D13"/>
-    <ns0:mergeCell ref="B14:D14"/>
-    <ns0:mergeCell ref="B15:D15"/>
-  </ns0:mergeCells>
-  <ns0:hyperlinks>
-    <ns0:hyperlink ref="B17" r:id="rId1"/>
-    <ns0:hyperlink ref="B18" r:id="rId2"/>
-    <ns0:hyperlink ref="B19" r:id="rId3"/>
-    <ns0:hyperlink ref="B20" r:id="rId4"/>
-    <ns0:hyperlink ref="B21" r:id="rId5"/>
-    <ns0:hyperlink ref="B22" r:id="rId6"/>
-    <ns0:hyperlink ref="B23" r:id="rId7"/>
-    <ns0:hyperlink ref="B26" r:id="rId10"/>
-    <ns0:hyperlink ref="B27" r:id="rId11"/>
-    <ns0:hyperlink ref="B28" r:id="rId12"/>
-    <ns0:hyperlink ref="B29" r:id="rId13"/>
-    <ns0:hyperlink ref="B31" r:id="rId14"/>
-    <ns0:hyperlink ref="B32" r:id="rId15"/>
-  </ns0:hyperlinks>
-  <ns0:pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
-</ns0:worksheet>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <cols>
+    <col min="1" max="1" width="28" customWidth="1"/>
+    <col min="2" max="2" width="23" customWidth="1"/>
+    <col min="3" max="3" width="31" customWidth="1"/>
+    <col min="4" max="4" width="88" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VARSAYIMLAR, SINIRLAR VE FİYAT KAYNAKLARI</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Çalışma tarihi</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">08.10.2026; arama sonuçlarında görülen çevrimiçi liste fiyatları kullanılmıştır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adet varsayımları</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pano 1: 14 + 6 = 20 adet 18,5 kW pompa. Pano 2: 4 + 5 = 9 adet 5,5 kW pompa. Pano 3: 7 + 3 = 10 adet 5,5 kW fan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Motor koruması</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Motor başına tek Siemens 3RV2 motor koruma şalteri kullanılır; ayrı termik röle satırları kaldırılmıştır. Sürücüsüz Y/Δ devrelerinde motor akım ayarı ve koordinasyon mühendislik hesabıyla doğrulanmalıdır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VFD + zaman rölesi</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bu tabloda zaman rölesi yıldız-üçgen için değil, VFD motorlarının kademeli devreye alınması için ek bütçe kalemidir; sürücünün dahili hızlanma rampası vardır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Zaman rölesi</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ENDA ATSP4 bağlantısı genel amaçlı analog zaman rölesi ürün sayfasıdır. Yıldız-üçgen işlev/çıkış kontak düzeni ve bobin gerilimi proje öncesi üretici dokümanından doğrulanmalıdır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kontrol/IO</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Waveshare 8DI/8DO kartı kullanıcı varsayımıyla mevcut kabul edilmiş ve maliyeti 0 TL yazılmıştır. 16 kanallı Modbus röle kartları 16 çıkış/motor kontaktör bobinleri varsayımıyla sayılmıştır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Eksik kontrol kalemi</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gerekli dijital giriş sayısı 8DI kapasitesini aşar; dijital giriş genişletmesi, haberleşme konfigürasyonu ve güvenli fail-safe tasarım maliyeti bu dosyada fiyatlandırılmamıştır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yıldız-üçgen emniyeti</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ESP32 zamanlaması tek başına emniyet değildir; yıldız/üçgen kontaktörlerinde mekanik kilitleme ve karşılıklı NC elektriksel kilitleme ile donanımsal acil-stop ve uygun motor koruma şalteri zinciri gerekir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kapsam dışı</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pano kabini, bara, kablolama, klemens, fan/filtre, SPD, ana kumanda/koruma aksesuarları, saha mühendisliği, montaj, devreye alma, nakliye ve işçilik toplamda yoktur. Liste tam satın alma BOM’u/uygulama projesi değildir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Teknik onay</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Motor etiket akımı, kısa devre seviyesi, koordinasyon, Siemens motor koruma şalteri ayar aralığı, sürücü giriş koruması, ana şalter seçimi ve pano ısıl hesabı yetkili elektrik mühendisi tarafından doğrulanmalıdır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fiyat/KDV</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Birim maliyetler TRY cinsindedir. Waveshare kart fiyatları kullanıcı tarafından belirtilmiştir (ESP32-S3 kartı 4.000 TL/adet; 16 kanal röle kartı 6.400 TL/adet). Diğer fiyatların KDV/iskonto durumu satıcıya göre değişir; toplamlar ön bütçedir, teklif değildir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stok / fiyat</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MPCB bağlantıları Siemens ürün kataloğuna gider; Türkiye satıcılarından fiyat/teslimat teklifi alınmalıdır. Güncel satıcı stoku ve KDV dahil fiyat teyit edilmediğinden motor koruma şalteri fiyatları ve pano toplamları “Teklif gerekli” görünür.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bara boyutlandırma</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ön BOM varsayımı: 18,5 kW pano için 30×10 mm paralel faz baraları; 5,5 kW panolar için 20×5 mm faz baraları ve PE barası. Kesit/paralel sayısı, bara mesafesi, destek/izolasyon, sıcaklık artışı, kısa devre dayanımı ve IEC 61439 uygunluğu yetkili elektrik mühendisi tarafından hesaplanıp doğrulanmalıdır; bu satırlar kesin proje/uygulama onayı değildir. Fiyatlar yaklaşık ve KDV/işleme/kargo durumu teyit edilmelidir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kalem</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Satıcı sayfası</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fiyata esas alınan tutar</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">18,5 kW Delta sürücü</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ürün sayfası</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">45.441,00 TL/adet</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sayhan çevrimiçi fiyatı; stok kontrolü gerekli.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1000 A kompakt şalter</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ürün sayfası</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">121.951,64 TL/adet</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tümpa liste fiyatı.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">160 A kompakt şalter</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ürün sayfası</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4.530,79 TL/adet</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tümpa fiyatı + KDV olarak raporlandı.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40 A motor koruma şalteri</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ürün sayfası</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5.946,48 TL/adet (KDV dahil listelenen fiyat)</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kullanıcının verdiği Elektrix ürünü: Siemens SIRIUS 3RV2021-4FA10, 34–40 A, 20 kA, S0; raya montajlı ve vidalı bağlantılı. Ürün liste sayfasındaki stok/fiyat siparişten önce teyit edilmeli; motor etiket akımı mühendis tarafından doğrulanmalı.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5,5 kW motor koruma şalteri</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ürün sayfası</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Teklif gerekli</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Siemens 3RV2011-1KA10, 9–12,5 A; 3RV2 S00, vidalı bağlantı, raya montaj. Üretici kataloğu; fiyat için Türkiye satıcı teklifi gerekli.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40 A / 18,5 kW kontaktör</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ürün sayfası</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5.170,00 TL/adet</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tümpa Siemens 24 V DC bobinli model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Siemens 3RT2017-1BB41, 12 A / 5,5 kW kontaktör</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ürün sayfası</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.137,00 TL/adet + KDV</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Elpimshop ürün sayfası; stokta 10+ adet bilgisi arama anında listelenmiş. Bobin 24 V DC, 1NA; stok ve fiyatı sipariş öncesi teyit edin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Eski 40 A termik röle</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kullanılmıyor; ilgili termik röle satırları Siemens motor koruma şalteriyle tek cihazda birleştirildi.</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ayrı termik röle kullanılmıyor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Eski 18 A termik röle</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kullanılmıyor; ilgili termik röle satırları Siemens motor koruma şalteriyle tek cihazda birleştirildi.</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ayrı termik röle kullanılmıyor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Analog zaman rölesi</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ürün sayfası</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.039,50 TL/adet</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sayhan indirimli fiyat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">24 V / 10 A güç kaynağı</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ürün sayfası</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2.062,84 TL/adet</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huzur Elektromarket fiyatı + KDV olarak raporlandı.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Waveshare 16 kanallı Modbus Ethernet röle kartı</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ürün sayfası</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6.400,00 TL/adet (kullanıcı tarafından belirtilen)</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kullanıcı tarafından verilen birim fiyat; Waveshare ürün sayfasından model/tedarik uygunluğu teyit edin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Waveshare ESP32-S3-POE-ETH-8DI-8DO</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ürün sayfası</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4.000,00 TL/adet (kullanıcı tarafından belirtilen)</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kullanıcı tarafından verilen birim fiyat; Waveshare ürün sayfasından model/tedarik uygunluğu teyit edin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bakır bara 30×10 mm × 3 m</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ürün sayfası</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">≈ 5.900 TL/bar</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hepsiburada listelemesi; arama anında yaklaşık ürün fiyatı. Liste seçeneği ve uzunluk/fiyatı sipariş öncesi teyit edin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bakır bara 20×5 mm × 1 m</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ürün sayfası</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">≈ 1.800 TL/bar</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hepsiburada ürün listesi; boy ve güncel fiyatı satın almadan önce teyit edin.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B15:D15"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="B17" r:id="rId1"/>
+    <hyperlink ref="B18" r:id="rId2"/>
+    <hyperlink ref="B19" r:id="rId3"/>
+    <hyperlink ref="B20" r:id="rId4"/>
+    <hyperlink ref="B21" r:id="rId5"/>
+    <hyperlink ref="B22" r:id="rId6"/>
+    <hyperlink ref="B23" r:id="rId7"/>
+    <hyperlink ref="B26" r:id="rId10"/>
+    <hyperlink ref="B27" r:id="rId11"/>
+    <hyperlink ref="B28" r:id="rId12"/>
+    <hyperlink ref="B29" r:id="rId13"/>
+    <hyperlink ref="B31" r:id="rId14"/>
+    <hyperlink ref="B32" r:id="rId15"/>
+  </hyperlinks>
+  <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add supplied Siemens protection and contactor prices
Co-authored-by: XDWOLLEN <74133863+XDWOLLEN@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/pano_varyasyon_maliyet.xlsx
+++ b/pano_varyasyon_maliyet.xlsx
@@ -1087,7 +1087,7 @@
     <ns0:row r="25">
       <ns0:c r="A25" s="5" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">Siemens SIRIUS 3RV2011-1KA10, 9–12,5 A motor koruma şalteri (vidalı bağlantı, DIN rayı)</ns0:t>
+          <ns0:t xml:space="preserve">Siemens SIRIUS 3RV2021-1KA10, 9–12,5 A motor koruma şalteri (KRC Elektrik)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="B25" s="6" t="inlineStr">
@@ -1095,10 +1095,8 @@
           <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="C25" s="8" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Teklif gerekli</ns0:t>
-        </ns0:is>
+      <ns0:c r="C25" s="8">
+        <ns0:v>6099.0</ns0:v>
       </ns0:c>
       <ns0:c r="D25" s="5">
         <ns0:v>9</ns0:v>
@@ -1109,7 +1107,7 @@
       </ns0:c>
       <ns0:c r="G25" s="5" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">Siemens SIRIUS 3RV2011-1KA10, 9–12,5 A motor koruma şalteri (vidalı bağlantı, DIN rayı)</ns0:t>
+          <ns0:t xml:space="preserve">Siemens SIRIUS 3RV2021-1KA10, 9–12,5 A motor koruma şalteri (KRC Elektrik)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="H25" s="6" t="inlineStr">
@@ -1117,10 +1115,8 @@
           <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="I25" s="8" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Teklif gerekli</ns0:t>
-        </ns0:is>
+      <ns0:c r="I25" s="8">
+        <ns0:v>6099.0</ns0:v>
       </ns0:c>
       <ns0:c r="J25" s="5">
         <ns0:v>9</ns0:v>
@@ -1141,10 +1137,8 @@
           <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="C26" s="8" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Teklif gerekli</ns0:t>
-        </ns0:is>
+      <ns0:c r="C26" s="8">
+        <ns0:v>1230.95</ns0:v>
       </ns0:c>
       <ns0:c r="D26" s="5">
         <ns0:v>27</ns0:v>
@@ -1163,10 +1157,8 @@
           <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="I26" s="8" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Teklif gerekli</ns0:t>
-        </ns0:is>
+      <ns0:c r="I26" s="8">
+        <ns0:v>1230.95</ns0:v>
       </ns0:c>
       <ns0:c r="J26" s="5">
         <ns0:v>27</ns0:v>
@@ -1505,7 +1497,7 @@
     <ns0:row r="42">
       <ns0:c r="A42" s="5" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">Siemens SIRIUS 3RV2011-1KA10, 9–12,5 A motor koruma şalteri (vidalı bağlantı, DIN rayı)</ns0:t>
+          <ns0:t xml:space="preserve">Siemens SIRIUS 3RV2021-1KA10, 9–12,5 A motor koruma şalteri (KRC Elektrik)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="B42" s="6" t="inlineStr">
@@ -1513,10 +1505,8 @@
           <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="C42" s="8" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Teklif gerekli</ns0:t>
-        </ns0:is>
+      <ns0:c r="C42" s="8">
+        <ns0:v>6099.0</ns0:v>
       </ns0:c>
       <ns0:c r="D42" s="5">
         <ns0:v>10</ns0:v>
@@ -1527,7 +1517,7 @@
       </ns0:c>
       <ns0:c r="G42" s="5" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">Siemens SIRIUS 3RV2011-1KA10, 9–12,5 A motor koruma şalteri (vidalı bağlantı, DIN rayı)</ns0:t>
+          <ns0:t xml:space="preserve">Siemens SIRIUS 3RV2021-1KA10, 9–12,5 A motor koruma şalteri (KRC Elektrik)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="H42" s="6" t="inlineStr">
@@ -1535,10 +1525,8 @@
           <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="I42" s="8" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Teklif gerekli</ns0:t>
-        </ns0:is>
+      <ns0:c r="I42" s="8">
+        <ns0:v>6099.0</ns0:v>
       </ns0:c>
       <ns0:c r="J42" s="5">
         <ns0:v>10</ns0:v>
@@ -1559,10 +1547,8 @@
           <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="C43" s="8" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Teklif gerekli</ns0:t>
-        </ns0:is>
+      <ns0:c r="C43" s="8">
+        <ns0:v>1230.95</ns0:v>
       </ns0:c>
       <ns0:c r="D43" s="5">
         <ns0:v>30</ns0:v>
@@ -1581,10 +1567,8 @@
           <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="I43" s="8" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Teklif gerekli</ns0:t>
-        </ns0:is>
+      <ns0:c r="I43" s="8">
+        <ns0:v>1230.95</ns0:v>
       </ns0:c>
       <ns0:c r="J43" s="5">
         <ns0:v>30</ns0:v>
@@ -2174,22 +2158,22 @@
     <ns0:row r="21">
       <ns0:c r="A21" s="5" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">5,5 kW motor koruma şalteri</ns0:t>
+          <ns0:t xml:space="preserve">Siemens 3RV2021-1KA10, 9–12,5 A motor koruma şalteri</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="B21" s="6" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">Ürün sayfası</ns0:t>
+          <ns0:t xml:space="preserve">KRC ürün sayfası</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="C21" s="5" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">Teklif gerekli</ns0:t>
+          <ns0:t xml:space="preserve">6.099,00 TL/adet (karşılaştırma fiyatı)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D21" s="5" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">Siemens 3RV2011-1KA10, 9–12,5 A; 3RV2 S00, vidalı bağlantı, raya montaj. Üretici kataloğu; fiyat için Türkiye satıcı teklifi gerekli.</ns0:t>
+          <ns0:t xml:space="preserve">Kullanıcının verdiği KRC ürün kodu/linki kullanıldı. KRC sayfasının fiyatı bu ortamdan okunamadı; aynı model için Santral Türkiye liste fiyatı 6.099 TL/adet olarak kullanılmıştır. KRC fiyatı ve stok sipariş öncesi teyit edilmeli.</ns0:t>
         </ns0:is>
       </ns0:c>
     </ns0:row>
@@ -2228,12 +2212,12 @@
       </ns0:c>
       <ns0:c r="C23" s="5" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">Teklif gerekli</ns0:t>
+          <ns0:t xml:space="preserve">1.230,95 TL/adet</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D23" s="5" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">Kullanıcının verdiği Zeybek Market ürün sayfası. Bobin gerilimi/ürün kodu ve güncel fiyatı erişim sırasında teyit edilemedi; sipariş öncesi teknik kod ve stok teyit edilmeli.</ns0:t>
+          <ns0:t xml:space="preserve">Zeybek Market ürün listeleme aramasında görülen güncel satış fiyatı; ürün sayfası bu dosyadan doğrudan açılamadı. Ürün kodu, bobin gerilimi, KDV ve stok sipariş öncesi teyit edilmeli.</ns0:t>
         </ns0:is>
       </ns0:c>
     </ns0:row>
@@ -2410,6 +2394,28 @@
       <ns0:c r="D32" s="5" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">Loobar ürün ailesi ve teknik bilgi kaynağı; belirli LB.4409.250 ürününün Türkiye stok ve fiyatı ayrıca teyit edilmeli.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="33">
+      <ns0:c r="A33" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Santral fiyat referansı — Siemens 3RV2021-1KA10</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B33" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Aynı model fiyatı</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C33" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">6.099,00 TL/adet</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D33" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">KRC sayfası fiyatı araç tarafından okunamadığı için kullanılan aynı model Türkiye satıcı referansı.</ns0:t>
         </ns0:is>
       </ns0:c>
     </ns0:row>
@@ -2444,6 +2450,7 @@
     <ns0:hyperlink ref="B29" r:id="rId13"/>
     <ns0:hyperlink ref="B31" r:id="rId14"/>
     <ns0:hyperlink ref="B32" r:id="rId15"/>
+    <ns0:hyperlink ref="B33" r:id="rId16"/>
   </ns0:hyperlinks>
   <ns0:pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </ns0:worksheet>

</xml_diff>

<commit_message>
Restore previous workbook formatting
Co-authored-by: XDWOLLEN <74133863+XDWOLLEN@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/pano_varyasyon_maliyet.xlsx
+++ b/pano_varyasyon_maliyet.xlsx
@@ -15,37 +15,44 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0.00 &quot;TL&quot;"/>
+    <numFmt numFmtId="164" formatCode="#,##0.00 &quot;₺&quot;"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
+      <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <bold>1</bold>
-      <sz>16</sz>
-      <color>FFFFFF</color>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <bold>1</bold>
-      <sz>10</sz>
-      <color>FFFFFF</color>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FF555555"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <bold>1</bold>
-      <sz>11</sz>
-      <color>FFFFFF</color>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <color>0563C1</color>
-      <underline>single</underline>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0563C1"/>
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -66,25 +73,37 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD9EAF7"/>
+        <fgColor rgb="FF4472C4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2F0D9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
   <borders count="2">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left style="thin">
-        <color rgb="FFB7C9D6"/>
+        <color rgb="FFD9E2F3"/>
       </left>
       <right style="thin">
-        <color rgb="FFB7C9D6"/>
+        <color rgb="FFD9E2F3"/>
       </right>
       <top style="thin">
-        <color rgb="FFB7C9D6"/>
+        <color rgb="FFD9E2F3"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFB7C9D6"/>
+        <color rgb="FFD9E2F3"/>
       </bottom>
       <diagonal/>
     </border>
@@ -94,35 +113,29 @@
   </cellStyleXfs>
   <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyAlignment="1" applyFont="1" applyFill="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFill="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFill="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFill="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyNumberFormat="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyNumberFormat="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyNumberFormat="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyAlignment="1" applyFont="1" applyFill="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="0" xfId="0" applyAlignment="1" applyFont="1" applyFill="1" applyNumberFormat="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -132,7 +145,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="20"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -201,13 +214,13 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C6" s="7">
+      <c r="C6" s="8">
         <v>121951.64</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="9">
         <v>1</v>
       </c>
-      <c r="E6" s="9">
+      <c r="E6" s="8">
         <f>IF(ISNUMBER(C6),C6*D6,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -223,13 +236,13 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C7" s="7">
+      <c r="C7" s="8">
         <v>5946.48</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="9">
         <v>20</v>
       </c>
-      <c r="E7" s="9">
+      <c r="E7" s="8">
         <f>IF(ISNUMBER(C7),C7*D7,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -245,13 +258,13 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C8" s="7">
+      <c r="C8" s="8">
         <v>45441.0</v>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="9">
         <v>20</v>
       </c>
-      <c r="E8" s="9">
+      <c r="E8" s="8">
         <f>IF(ISNUMBER(C8),C8*D8,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -267,13 +280,13 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C9" s="7">
+      <c r="C9" s="8">
         <v>2062.84</v>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="9">
         <v>1</v>
       </c>
-      <c r="E9" s="9">
+      <c r="E9" s="8">
         <f>IF(ISNUMBER(C9),C9*D9,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -289,13 +302,13 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C10" s="7">
+      <c r="C10" s="8">
         <v>4000.0</v>
       </c>
-      <c r="D10" s="8">
+      <c r="D10" s="9">
         <v>1</v>
       </c>
-      <c r="E10" s="9">
+      <c r="E10" s="8">
         <f>IF(ISNUMBER(C10),C10*D10,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -311,13 +324,13 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C11" s="7">
+      <c r="C11" s="8">
         <v>6400.0</v>
       </c>
-      <c r="D11" s="8">
+      <c r="D11" s="9">
         <v>2</v>
       </c>
-      <c r="E11" s="9">
+      <c r="E11" s="8">
         <f>IF(ISNUMBER(C11),C11*D11,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -338,10 +351,10 @@
           <t>Teklif gerekli</t>
         </is>
       </c>
-      <c r="D12" s="8">
+      <c r="D12" s="9">
         <v>4</v>
       </c>
-      <c r="E12" s="9">
+      <c r="E12" s="8">
         <f>IF(ISNUMBER(C12),C12*D12,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -369,7 +382,7 @@
       </c>
     </row>
     <row r="15" ht="21" customHeight="1">
-      <c r="A15" s="12" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Teknik not: VFD çıkışında yıldız-üçgen kontaktör geçişi/zaman rölesi kullanılmaz. Motor, etiketine göre sabit yıldız veya üçgen bağlanır; hızlanma rampası sürücüden ayarlanır. Bu nedenle Pano 1 listesine Y/Δ zaman rölesi ve Y/Δ kontaktörleri eklenmemiştir.</t>
         </is>
@@ -420,13 +433,13 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C19" s="7">
+      <c r="C19" s="8">
         <v>4530.79</v>
       </c>
-      <c r="D19" s="8">
+      <c r="D19" s="9">
         <v>1</v>
       </c>
-      <c r="E19" s="9">
+      <c r="E19" s="8">
         <f>IF(ISNUMBER(C19),C19*D19,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -442,13 +455,13 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C20" s="7">
+      <c r="C20" s="8">
         <v>6099.0</v>
       </c>
-      <c r="D20" s="8">
+      <c r="D20" s="9">
         <v>9</v>
       </c>
-      <c r="E20" s="9">
+      <c r="E20" s="8">
         <f>IF(ISNUMBER(C20),C20*D20,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -464,13 +477,13 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C21" s="7">
+      <c r="C21" s="8">
         <v>1230.95</v>
       </c>
-      <c r="D21" s="8">
+      <c r="D21" s="9">
         <v>27</v>
       </c>
-      <c r="E21" s="9">
+      <c r="E21" s="8">
         <f>IF(ISNUMBER(C21),C21*D21,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -486,13 +499,13 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C22" s="7">
+      <c r="C22" s="8">
         <v>1039.5</v>
       </c>
-      <c r="D22" s="8">
+      <c r="D22" s="9">
         <v>9</v>
       </c>
-      <c r="E22" s="9">
+      <c r="E22" s="8">
         <f>IF(ISNUMBER(C22),C22*D22,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -508,13 +521,13 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C23" s="7">
+      <c r="C23" s="8">
         <v>2062.84</v>
       </c>
-      <c r="D23" s="8">
+      <c r="D23" s="9">
         <v>1</v>
       </c>
-      <c r="E23" s="9">
+      <c r="E23" s="8">
         <f>IF(ISNUMBER(C23),C23*D23,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -530,13 +543,13 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C24" s="7">
+      <c r="C24" s="8">
         <v>4000.0</v>
       </c>
-      <c r="D24" s="8">
+      <c r="D24" s="9">
         <v>1</v>
       </c>
-      <c r="E24" s="9">
+      <c r="E24" s="8">
         <f>IF(ISNUMBER(C24),C24*D24,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -552,13 +565,13 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C25" s="7">
+      <c r="C25" s="8">
         <v>6400.0</v>
       </c>
-      <c r="D25" s="8">
+      <c r="D25" s="9">
         <v>2</v>
       </c>
-      <c r="E25" s="9">
+      <c r="E25" s="8">
         <f>IF(ISNUMBER(C25),C25*D25,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -579,10 +592,10 @@
           <t>Teklif gerekli</t>
         </is>
       </c>
-      <c r="D26" s="8">
+      <c r="D26" s="9">
         <v>1</v>
       </c>
-      <c r="E26" s="9">
+      <c r="E26" s="8">
         <f>IF(ISNUMBER(C26),C26*D26,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -610,7 +623,7 @@
       </c>
     </row>
     <row r="29" ht="21" customHeight="1">
-      <c r="A29" s="12" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>Her pompa için 1 motor koruma şalteri, 3 adet Siemens kontaktör ve 1 yıldız-üçgen zaman rölesi varsayılmıştır. Y/Δ kontaktörlerinde uygun mekanik ve elektriksel kilitleme zorunludur.</t>
         </is>
@@ -661,13 +674,13 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C33" s="7">
+      <c r="C33" s="8">
         <v>4530.79</v>
       </c>
-      <c r="D33" s="8">
+      <c r="D33" s="9">
         <v>1</v>
       </c>
-      <c r="E33" s="9">
+      <c r="E33" s="8">
         <f>IF(ISNUMBER(C33),C33*D33,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -683,13 +696,13 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C34" s="7">
+      <c r="C34" s="8">
         <v>6099.0</v>
       </c>
-      <c r="D34" s="8">
+      <c r="D34" s="9">
         <v>10</v>
       </c>
-      <c r="E34" s="9">
+      <c r="E34" s="8">
         <f>IF(ISNUMBER(C34),C34*D34,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -705,13 +718,13 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C35" s="7">
+      <c r="C35" s="8">
         <v>1230.95</v>
       </c>
-      <c r="D35" s="8">
+      <c r="D35" s="9">
         <v>30</v>
       </c>
-      <c r="E35" s="9">
+      <c r="E35" s="8">
         <f>IF(ISNUMBER(C35),C35*D35,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -727,13 +740,13 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C36" s="7">
+      <c r="C36" s="8">
         <v>1039.5</v>
       </c>
-      <c r="D36" s="8">
+      <c r="D36" s="9">
         <v>10</v>
       </c>
-      <c r="E36" s="9">
+      <c r="E36" s="8">
         <f>IF(ISNUMBER(C36),C36*D36,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -749,13 +762,13 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C37" s="7">
+      <c r="C37" s="8">
         <v>2062.84</v>
       </c>
-      <c r="D37" s="8">
+      <c r="D37" s="9">
         <v>1</v>
       </c>
-      <c r="E37" s="9">
+      <c r="E37" s="8">
         <f>IF(ISNUMBER(C37),C37*D37,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -771,13 +784,13 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C38" s="7">
+      <c r="C38" s="8">
         <v>4000.0</v>
       </c>
-      <c r="D38" s="8">
+      <c r="D38" s="9">
         <v>1</v>
       </c>
-      <c r="E38" s="9">
+      <c r="E38" s="8">
         <f>IF(ISNUMBER(C38),C38*D38,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -793,13 +806,13 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C39" s="7">
+      <c r="C39" s="8">
         <v>6400.0</v>
       </c>
-      <c r="D39" s="8">
+      <c r="D39" s="9">
         <v>2</v>
       </c>
-      <c r="E39" s="9">
+      <c r="E39" s="8">
         <f>IF(ISNUMBER(C39),C39*D39,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -820,10 +833,10 @@
           <t>Teklif gerekli</t>
         </is>
       </c>
-      <c r="D40" s="8">
+      <c r="D40" s="9">
         <v>1</v>
       </c>
-      <c r="E40" s="9">
+      <c r="E40" s="8">
         <f>IF(ISNUMBER(C40),C40*D40,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -851,7 +864,7 @@
       </c>
     </row>
     <row r="43" ht="21" customHeight="1">
-      <c r="A43" s="12" t="inlineStr">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>Her fan motoru için 1 motor koruma şalteri, 3 adet Siemens kontaktör ve 1 yıldız-üçgen zaman rölesi varsayılmıştır. Y/Δ kontaktörlerinde uygun mekanik ve elektriksel kilitleme zorunludur.</t>
         </is>
@@ -902,13 +915,13 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C47" s="8">
+      <c r="C47" s="9">
         <v>1</v>
       </c>
-      <c r="D47" s="7">
+      <c r="D47" s="8">
         <v>121951.64</v>
       </c>
-      <c r="E47" s="9">
+      <c r="E47" s="8">
         <f>IF(ISNUMBER(D47),C47*D47,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -924,13 +937,13 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C48" s="8">
+      <c r="C48" s="9">
         <v>20</v>
       </c>
-      <c r="D48" s="7">
+      <c r="D48" s="8">
         <v>5946.48</v>
       </c>
-      <c r="E48" s="9">
+      <c r="E48" s="8">
         <f>IF(ISNUMBER(D48),C48*D48,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -946,13 +959,13 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C49" s="8">
+      <c r="C49" s="9">
         <v>20</v>
       </c>
-      <c r="D49" s="7">
+      <c r="D49" s="8">
         <v>45441.0</v>
       </c>
-      <c r="E49" s="9">
+      <c r="E49" s="8">
         <f>IF(ISNUMBER(D49),C49*D49,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -968,13 +981,13 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C50" s="8">
+      <c r="C50" s="9">
         <v>3</v>
       </c>
-      <c r="D50" s="7">
+      <c r="D50" s="8">
         <v>2062.84</v>
       </c>
-      <c r="E50" s="9">
+      <c r="E50" s="8">
         <f>IF(ISNUMBER(D50),C50*D50,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -990,13 +1003,13 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C51" s="8">
+      <c r="C51" s="9">
         <v>3</v>
       </c>
-      <c r="D51" s="7">
+      <c r="D51" s="8">
         <v>4000.0</v>
       </c>
-      <c r="E51" s="9">
+      <c r="E51" s="8">
         <f>IF(ISNUMBER(D51),C51*D51,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -1012,13 +1025,13 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C52" s="8">
+      <c r="C52" s="9">
         <v>6</v>
       </c>
-      <c r="D52" s="7">
+      <c r="D52" s="8">
         <v>6400.0</v>
       </c>
-      <c r="E52" s="9">
+      <c r="E52" s="8">
         <f>IF(ISNUMBER(D52),C52*D52,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -1034,7 +1047,7 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C53" s="8">
+      <c r="C53" s="9">
         <v>6</v>
       </c>
       <c r="D53" s="5" t="inlineStr">
@@ -1042,7 +1055,7 @@
           <t>Teklif gerekli</t>
         </is>
       </c>
-      <c r="E53" s="9">
+      <c r="E53" s="8">
         <f>IF(ISNUMBER(D53),C53*D53,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -1058,13 +1071,13 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C54" s="8">
+      <c r="C54" s="9">
         <v>2</v>
       </c>
-      <c r="D54" s="7">
+      <c r="D54" s="8">
         <v>4530.79</v>
       </c>
-      <c r="E54" s="9">
+      <c r="E54" s="8">
         <f>IF(ISNUMBER(D54),C54*D54,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -1080,13 +1093,13 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C55" s="8">
+      <c r="C55" s="9">
         <v>19</v>
       </c>
-      <c r="D55" s="7">
+      <c r="D55" s="8">
         <v>6099.0</v>
       </c>
-      <c r="E55" s="9">
+      <c r="E55" s="8">
         <f>IF(ISNUMBER(D55),C55*D55,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -1102,13 +1115,13 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C56" s="8">
+      <c r="C56" s="9">
         <v>57</v>
       </c>
-      <c r="D56" s="7">
+      <c r="D56" s="8">
         <v>1230.95</v>
       </c>
-      <c r="E56" s="9">
+      <c r="E56" s="8">
         <f>IF(ISNUMBER(D56),C56*D56,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -1124,13 +1137,13 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C57" s="8">
+      <c r="C57" s="9">
         <v>19</v>
       </c>
-      <c r="D57" s="7">
+      <c r="D57" s="8">
         <v>1039.5</v>
       </c>
-      <c r="E57" s="9">
+      <c r="E57" s="8">
         <f>IF(ISNUMBER(D57),C57*D57,"Teklif gerekli")</f>
         <v/>
       </c>
@@ -1158,7 +1171,7 @@
       </c>
     </row>
     <row r="60" ht="21" customHeight="1">
-      <c r="A60" s="12" t="inlineStr">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>“Teklif gerekli” kalemin bedeli, ara toplamda yer almaz; nihai satın alma toplamı satıcı teklifiyle tamamlanmalıdır.</t>
         </is>
@@ -1186,47 +1199,47 @@
     <mergeCell ref="A60:E60"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B6" r:id="rId1"/>
-    <hyperlink ref="B7" r:id="rId2"/>
-    <hyperlink ref="B8" r:id="rId3"/>
-    <hyperlink ref="B9" r:id="rId4"/>
-    <hyperlink ref="B10" r:id="rId5"/>
-    <hyperlink ref="B11" r:id="rId6"/>
-    <hyperlink ref="B12" r:id="rId7"/>
-    <hyperlink ref="B19" r:id="rId8"/>
-    <hyperlink ref="B20" r:id="rId9"/>
-    <hyperlink ref="B21" r:id="rId10"/>
-    <hyperlink ref="B22" r:id="rId11"/>
-    <hyperlink ref="B23" r:id="rId4"/>
-    <hyperlink ref="B24" r:id="rId5"/>
-    <hyperlink ref="B25" r:id="rId6"/>
-    <hyperlink ref="B26" r:id="rId7"/>
-    <hyperlink ref="B33" r:id="rId8"/>
-    <hyperlink ref="B34" r:id="rId9"/>
-    <hyperlink ref="B35" r:id="rId10"/>
-    <hyperlink ref="B36" r:id="rId11"/>
-    <hyperlink ref="B37" r:id="rId4"/>
-    <hyperlink ref="B38" r:id="rId5"/>
-    <hyperlink ref="B39" r:id="rId6"/>
-    <hyperlink ref="B40" r:id="rId7"/>
-    <hyperlink ref="B47" r:id="rId1"/>
-    <hyperlink ref="B48" r:id="rId2"/>
-    <hyperlink ref="B49" r:id="rId3"/>
-    <hyperlink ref="B50" r:id="rId4"/>
-    <hyperlink ref="B51" r:id="rId5"/>
-    <hyperlink ref="B52" r:id="rId6"/>
-    <hyperlink ref="B53" r:id="rId7"/>
-    <hyperlink ref="B54" r:id="rId8"/>
-    <hyperlink ref="B55" r:id="rId9"/>
-    <hyperlink ref="B56" r:id="rId10"/>
-    <hyperlink ref="B57" r:id="rId11"/>
+    <hyperlink ref="B6" ns1:id="rId1"/>
+    <hyperlink ref="B7" ns1:id="rId2"/>
+    <hyperlink ref="B8" ns1:id="rId3"/>
+    <hyperlink ref="B9" ns1:id="rId4"/>
+    <hyperlink ref="B10" ns1:id="rId5"/>
+    <hyperlink ref="B11" ns1:id="rId6"/>
+    <hyperlink ref="B12" ns1:id="rId7"/>
+    <hyperlink ref="B19" ns1:id="rId8"/>
+    <hyperlink ref="B20" ns1:id="rId9"/>
+    <hyperlink ref="B21" ns1:id="rId10"/>
+    <hyperlink ref="B22" ns1:id="rId11"/>
+    <hyperlink ref="B23" ns1:id="rId4"/>
+    <hyperlink ref="B24" ns1:id="rId5"/>
+    <hyperlink ref="B25" ns1:id="rId6"/>
+    <hyperlink ref="B26" ns1:id="rId7"/>
+    <hyperlink ref="B33" ns1:id="rId8"/>
+    <hyperlink ref="B34" ns1:id="rId9"/>
+    <hyperlink ref="B35" ns1:id="rId10"/>
+    <hyperlink ref="B36" ns1:id="rId11"/>
+    <hyperlink ref="B37" ns1:id="rId4"/>
+    <hyperlink ref="B38" ns1:id="rId5"/>
+    <hyperlink ref="B39" ns1:id="rId6"/>
+    <hyperlink ref="B40" ns1:id="rId7"/>
+    <hyperlink ref="B47" ns1:id="rId1"/>
+    <hyperlink ref="B48" ns1:id="rId2"/>
+    <hyperlink ref="B49" ns1:id="rId3"/>
+    <hyperlink ref="B50" ns1:id="rId4"/>
+    <hyperlink ref="B51" ns1:id="rId5"/>
+    <hyperlink ref="B52" ns1:id="rId6"/>
+    <hyperlink ref="B53" ns1:id="rId7"/>
+    <hyperlink ref="B54" ns1:id="rId8"/>
+    <hyperlink ref="B55" ns1:id="rId9"/>
+    <hyperlink ref="B56" ns1:id="rId10"/>
+    <hyperlink ref="B57" ns1:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="20"/>
   <cols>
     <col min="1" max="1" width="37" customWidth="1"/>
@@ -1255,7 +1268,7 @@
           <t>Motor adetleri</t>
         </is>
       </c>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Pano 1: 14 + 6 = 20 adet 18,5 kW pompa; Pano 2: 4 + 5 = 9 adet 5,5 kW pompa; Pano 3: 7 + 3 = 10 adet 5,5 kW fan.</t>
         </is>
@@ -1267,7 +1280,7 @@
           <t>Pano 1 tasarımı</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>20 adet 18,5 kW VFD baz alınmıştır. Y/Δ geçişi için zaman rölesi eklenmemiştir: VFD ile motor arasında çalışma sırasında yıldız-üçgen kontaktör geçişi sürücüye/motora zarar verebilir. Motor sabit bağlantıda kalmalı; rampa sürücüden ayarlanmalıdır.</t>
         </is>
@@ -1279,7 +1292,7 @@
           <t>Pano 2 ve 3</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Her 5,5 kW motor için 1 adet motor koruma şalteri, 3 Siemens kontaktör ve 1 zaman rölesi öngörülmüştür. Kontaktör yıldız/ana/üçgen görevleri, bobin gerilimi, kontaktör boyutlandırması ve zaman rölesinin gerçek Y/Δ fonksiyonu üretici dokümanı/proje ile doğrulanmalıdır.</t>
         </is>
@@ -1291,7 +1304,7 @@
           <t>MPCB</t>
         </is>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Termik röle yerine raya montajlı Siemens 3RV2 motor koruma şalterleri listelenmiştir. Ayar aralığının motor etiket akımına uygunluğu ve sürücü öncesi koruma/koordinasyon yetkili elektrik mühendisi tarafından kontrol edilmelidir.</t>
         </is>
@@ -1303,7 +1316,7 @@
           <t>Waveshare kartları</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Kullanıcının verdiği fiyatlar kullanılmıştır: ESP32-S3-POE-ETH-8DI-8DO (mevcut) 4.000 TL/adet; 16 kanallı Modbus Ethernet röle kartı 6.400 TL/adet. Adetler mevcut tasarım kabulüdür; giriş/çıkış kapasitesi ve fail-safe kontrol ayrıca doğrulanmalıdır.</t>
         </is>
@@ -1315,7 +1328,7 @@
           <t>Loobar dağıtım kutusu</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>LB.4409.250 4 kutuplu 250 A güç dağıtım kutusu/barasıdır; bakır lama değildir. 18,5 kW pano için 4 ayrı grup, diğer panolar için birer adet ön seçimdir. Fiyat KRC ürün sayfasında teyit edilemediği için teklif gerekli bırakıldı; ara toplamlar bu kalemi içermez. PE/topraklama barası yerine geçmez.</t>
         </is>
@@ -1327,7 +1340,7 @@
           <t>Fiyat ve KDV</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Diğer birim fiyatlar önceki araştırmada görülen satıcı listeleme/karşılaştırma tutarlarıdır; KDV ve iskonto satıcı bazında farklı olabilir. Zeybek kontaktör ve KRC 12,5 A koruma şalteri fiyatları sipariş öncesi ürün kodu, stok ve güncel tutar açısından doğrulanmalıdır.</t>
         </is>
@@ -1339,7 +1352,7 @@
           <t>Kapsam dışı</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Pano kabini, ana bara/kablolama, klemensler, fan/filtre, SPD, kumanda/koruma aksesuarları, ilave giriş/çıkış genişlemesi, montaj, devreye alma, mühendislik, nakliye ve işçilik dahil değildir. Liste uygulama projesi yerine geçmez.</t>
         </is>
@@ -1351,7 +1364,7 @@
           <t>Toplamlar</t>
         </is>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Kalem toplamı = birim fiyat × miktar formülüdür. Pano ve toplu satın alma toplamı formüllerle hesaplanır. Teklif gereken satır olduğunda kesin toplam yerine fiyatı bilinen kalemlerin ara toplamı gösterilir.</t>
         </is>
@@ -1390,10 +1403,10 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C15" s="7">
+      <c r="C15" s="8">
         <v>121951.64</v>
       </c>
-      <c r="D15" s="12" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>Tümpa liste fiyatı.</t>
         </is>
@@ -1410,10 +1423,10 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C16" s="7">
+      <c r="C16" s="8">
         <v>5946.48</v>
       </c>
-      <c r="D16" s="12" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Elektrix; listelenen fiyat. Stok/fiyatı teyit edin.</t>
         </is>
@@ -1430,10 +1443,10 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C17" s="7">
+      <c r="C17" s="8">
         <v>45441.0</v>
       </c>
-      <c r="D17" s="12" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>Sayhan çevrimiçi fiyatı.</t>
         </is>
@@ -1450,10 +1463,10 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C18" s="7">
+      <c r="C18" s="8">
         <v>4530.79</v>
       </c>
-      <c r="D18" s="12" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Tümpa fiyatı + KDV olarak raporlandı.</t>
         </is>
@@ -1470,10 +1483,10 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C19" s="7">
+      <c r="C19" s="8">
         <v>6099.0</v>
       </c>
-      <c r="D19" s="12" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>KRC linki; KRC fiyatı okunamadığından aynı model karşılaştırma fiyatı kullanıldı.</t>
         </is>
@@ -1490,10 +1503,10 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C20" s="7">
+      <c r="C20" s="8">
         <v>1230.95</v>
       </c>
-      <c r="D20" s="12" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>Zeybek listeleme fiyatı; güncel ürün/kod/stok doğrulaması gerekli.</t>
         </is>
@@ -1510,10 +1523,10 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C21" s="7">
+      <c r="C21" s="8">
         <v>1039.5</v>
       </c>
-      <c r="D21" s="12" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>Sayhan indirimli fiyatı; Y/Δ fonksiyonunu teyit edin.</t>
         </is>
@@ -1530,10 +1543,10 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C22" s="7">
+      <c r="C22" s="8">
         <v>2062.84</v>
       </c>
-      <c r="D22" s="12" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>Huzur Elektromarket fiyatı + KDV olarak raporlandı.</t>
         </is>
@@ -1550,10 +1563,10 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C23" s="7">
+      <c r="C23" s="8">
         <v>4000.0</v>
       </c>
-      <c r="D23" s="12" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>Kullanıcının belirttiği fiyat.</t>
         </is>
@@ -1570,10 +1583,10 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C24" s="7">
+      <c r="C24" s="8">
         <v>6400.0</v>
       </c>
-      <c r="D24" s="12" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>Kullanıcının belirttiği fiyat.</t>
         </is>
@@ -1595,7 +1608,7 @@
           <t>Teklif gerekli</t>
         </is>
       </c>
-      <c r="D25" s="12" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>KRC ürün bağlantısı; güncel fiyat/stok teyit edilmedi, teklif gerekli.</t>
         </is>
@@ -1616,17 +1629,17 @@
     <mergeCell ref="B12:D12"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B15" r:id="rId1"/>
-    <hyperlink ref="B16" r:id="rId2"/>
-    <hyperlink ref="B17" r:id="rId3"/>
-    <hyperlink ref="B18" r:id="rId4"/>
-    <hyperlink ref="B19" r:id="rId5"/>
-    <hyperlink ref="B20" r:id="rId6"/>
-    <hyperlink ref="B21" r:id="rId7"/>
-    <hyperlink ref="B22" r:id="rId8"/>
-    <hyperlink ref="B23" r:id="rId9"/>
-    <hyperlink ref="B24" r:id="rId10"/>
-    <hyperlink ref="B25" r:id="rId11"/>
+    <hyperlink ref="B15" ns1:id="rId1"/>
+    <hyperlink ref="B16" ns1:id="rId2"/>
+    <hyperlink ref="B17" ns1:id="rId3"/>
+    <hyperlink ref="B18" ns1:id="rId4"/>
+    <hyperlink ref="B19" ns1:id="rId5"/>
+    <hyperlink ref="B20" ns1:id="rId6"/>
+    <hyperlink ref="B21" ns1:id="rId7"/>
+    <hyperlink ref="B22" ns1:id="rId8"/>
+    <hyperlink ref="B23" ns1:id="rId9"/>
+    <hyperlink ref="B24" ns1:id="rId10"/>
+    <hyperlink ref="B25" ns1:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 600A four-pole copper busbar to procurement list
Co-authored-by: XDWOLLEN <74133863+XDWOLLEN@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/pano_varyasyon_maliyet.xlsx
+++ b/pano_varyasyon_maliyet.xlsx
@@ -145,7 +145,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="20"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -1149,29 +1149,51 @@
       </c>
     </row>
     <row r="58" ht="21" customHeight="1">
-      <c r="A58" s="10" t="inlineStr">
-        <is>
-          <t>Fiyatı bilinen kalemler ara toplamı</t>
-        </is>
-      </c>
-      <c r="E58" s="11">
-        <f>SUM(E47:E57)</f>
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Loobar LB.4212.600, 4 kutuplu 600 A kalaylı bakır baralı dağıtıcı</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>Ürün sayfası</t>
+        </is>
+      </c>
+      <c r="C58" s="9">
+        <v>1</v>
+      </c>
+      <c r="D58" s="8">
+        <v>11816.92</v>
+      </c>
+      <c r="E58" s="8">
+        <f>IF(ISNUMBER(D58),C58*D58,"Teklif gerekli")</f>
         <v/>
       </c>
     </row>
     <row r="59" ht="21" customHeight="1">
       <c r="A59" s="10" t="inlineStr">
         <is>
+          <t>Fiyatı bilinen kalemler ara toplamı</t>
+        </is>
+      </c>
+      <c r="E59" s="11">
+        <f>SUM(E47:E58)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60" ht="21" customHeight="1">
+      <c r="A60" s="10" t="inlineStr">
+        <is>
           <t>Genel satın alma toplamı</t>
         </is>
       </c>
-      <c r="E59" s="11">
-        <f>IF(COUNT(E47:E57)&lt;COUNTA(A47:A57),"TEKLİF GEREKLİ",SUM(E47:E57))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60" ht="21" customHeight="1">
-      <c r="A60" s="2" t="inlineStr">
+      <c r="E60" s="11">
+        <f>IF(COUNT(E47:E58)&lt;COUNTA(A47:A58),"TEKLİF GEREKLİ",SUM(E47:E58))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61" ht="21" customHeight="1">
+      <c r="A61" s="2" t="inlineStr">
         <is>
           <t>“Teklif gerekli” kalemin bedeli, ara toplamda yer almaz; nihai satın alma toplamı satıcı teklifiyle tamamlanmalıdır.</t>
         </is>
@@ -1199,47 +1221,48 @@
     <mergeCell ref="A60:E60"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B6" ns1:id="rId1"/>
-    <hyperlink ref="B7" ns1:id="rId2"/>
-    <hyperlink ref="B8" ns1:id="rId3"/>
-    <hyperlink ref="B9" ns1:id="rId4"/>
-    <hyperlink ref="B10" ns1:id="rId5"/>
-    <hyperlink ref="B11" ns1:id="rId6"/>
-    <hyperlink ref="B12" ns1:id="rId7"/>
-    <hyperlink ref="B19" ns1:id="rId8"/>
-    <hyperlink ref="B20" ns1:id="rId9"/>
-    <hyperlink ref="B21" ns1:id="rId10"/>
-    <hyperlink ref="B22" ns1:id="rId11"/>
-    <hyperlink ref="B23" ns1:id="rId4"/>
-    <hyperlink ref="B24" ns1:id="rId5"/>
-    <hyperlink ref="B25" ns1:id="rId6"/>
-    <hyperlink ref="B26" ns1:id="rId7"/>
-    <hyperlink ref="B33" ns1:id="rId8"/>
-    <hyperlink ref="B34" ns1:id="rId9"/>
-    <hyperlink ref="B35" ns1:id="rId10"/>
-    <hyperlink ref="B36" ns1:id="rId11"/>
-    <hyperlink ref="B37" ns1:id="rId4"/>
-    <hyperlink ref="B38" ns1:id="rId5"/>
-    <hyperlink ref="B39" ns1:id="rId6"/>
-    <hyperlink ref="B40" ns1:id="rId7"/>
-    <hyperlink ref="B47" ns1:id="rId1"/>
-    <hyperlink ref="B48" ns1:id="rId2"/>
-    <hyperlink ref="B49" ns1:id="rId3"/>
-    <hyperlink ref="B50" ns1:id="rId4"/>
-    <hyperlink ref="B51" ns1:id="rId5"/>
-    <hyperlink ref="B52" ns1:id="rId6"/>
-    <hyperlink ref="B53" ns1:id="rId7"/>
-    <hyperlink ref="B54" ns1:id="rId8"/>
-    <hyperlink ref="B55" ns1:id="rId9"/>
-    <hyperlink ref="B56" ns1:id="rId10"/>
-    <hyperlink ref="B57" ns1:id="rId11"/>
+    <hyperlink ref="B6" r:id="rId1"/>
+    <hyperlink ref="B7" r:id="rId2"/>
+    <hyperlink ref="B8" r:id="rId3"/>
+    <hyperlink ref="B9" r:id="rId4"/>
+    <hyperlink ref="B10" r:id="rId5"/>
+    <hyperlink ref="B11" r:id="rId6"/>
+    <hyperlink ref="B12" r:id="rId7"/>
+    <hyperlink ref="B19" r:id="rId8"/>
+    <hyperlink ref="B20" r:id="rId9"/>
+    <hyperlink ref="B21" r:id="rId10"/>
+    <hyperlink ref="B22" r:id="rId11"/>
+    <hyperlink ref="B23" r:id="rId4"/>
+    <hyperlink ref="B24" r:id="rId5"/>
+    <hyperlink ref="B25" r:id="rId6"/>
+    <hyperlink ref="B26" r:id="rId7"/>
+    <hyperlink ref="B33" r:id="rId8"/>
+    <hyperlink ref="B34" r:id="rId9"/>
+    <hyperlink ref="B35" r:id="rId10"/>
+    <hyperlink ref="B36" r:id="rId11"/>
+    <hyperlink ref="B37" r:id="rId4"/>
+    <hyperlink ref="B38" r:id="rId5"/>
+    <hyperlink ref="B39" r:id="rId6"/>
+    <hyperlink ref="B40" r:id="rId7"/>
+    <hyperlink ref="B47" r:id="rId1"/>
+    <hyperlink ref="B48" r:id="rId2"/>
+    <hyperlink ref="B49" r:id="rId3"/>
+    <hyperlink ref="B50" r:id="rId4"/>
+    <hyperlink ref="B51" r:id="rId5"/>
+    <hyperlink ref="B52" r:id="rId6"/>
+    <hyperlink ref="B53" r:id="rId7"/>
+    <hyperlink ref="B54" r:id="rId8"/>
+    <hyperlink ref="B55" r:id="rId9"/>
+    <hyperlink ref="B56" r:id="rId10"/>
+    <hyperlink ref="B57" r:id="rId11"/>
+    <hyperlink ref="B58" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="20"/>
   <cols>
     <col min="1" max="1" width="37" customWidth="1"/>
@@ -1354,7 +1377,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Pano kabini, ana bara/kablolama, klemensler, fan/filtre, SPD, kumanda/koruma aksesuarları, ilave giriş/çıkış genişlemesi, montaj, devreye alma, mühendislik, nakliye ve işçilik dahil değildir. Liste uygulama projesi yerine geçmez.</t>
+          <t>Pano kabini, pano içi ana bara ve kablolama (toplu listeye ayrıca eklenen 600 A dağıtıcı hariç), klemensler, fan/filtre, SPD, kumanda/koruma aksesuarları, ilave giriş/çıkış genişlemesi, montaj, devreye alma, mühendislik, nakliye ve işçilik dahil değildir. Liste uygulama projesi yerine geçmez.</t>
         </is>
       </c>
     </row>
@@ -1611,6 +1634,26 @@
       <c r="D25" s="2" t="inlineStr">
         <is>
           <t>KRC ürün bağlantısı; güncel fiyat/stok teyit edilmedi, teklif gerekli.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Loobar LB.4212.600, 600 A bakır baralı dağıtıcı</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>Ürün sayfası</t>
+        </is>
+      </c>
+      <c r="C26" s="8">
+        <v>11816.92</v>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Loobar ürün sayfasında 11.816,92 TL + KDV liste fiyatı olarak görülen tutar; stok/fiyat sipariş öncesi teyit edilmeli. Toplu listede 1 adet geçici varsayımdır; pano bazlı adet belirtilmediği için pano BOM’larına eklenmedi.</t>
         </is>
       </c>
     </row>
@@ -1629,17 +1672,18 @@
     <mergeCell ref="B12:D12"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B15" ns1:id="rId1"/>
-    <hyperlink ref="B16" ns1:id="rId2"/>
-    <hyperlink ref="B17" ns1:id="rId3"/>
-    <hyperlink ref="B18" ns1:id="rId4"/>
-    <hyperlink ref="B19" ns1:id="rId5"/>
-    <hyperlink ref="B20" ns1:id="rId6"/>
-    <hyperlink ref="B21" ns1:id="rId7"/>
-    <hyperlink ref="B22" ns1:id="rId8"/>
-    <hyperlink ref="B23" ns1:id="rId9"/>
-    <hyperlink ref="B24" ns1:id="rId10"/>
-    <hyperlink ref="B25" ns1:id="rId11"/>
+    <hyperlink ref="B15" r:id="rId1"/>
+    <hyperlink ref="B16" r:id="rId2"/>
+    <hyperlink ref="B17" r:id="rId3"/>
+    <hyperlink ref="B18" r:id="rId4"/>
+    <hyperlink ref="B19" r:id="rId5"/>
+    <hyperlink ref="B20" r:id="rId6"/>
+    <hyperlink ref="B21" r:id="rId7"/>
+    <hyperlink ref="B22" r:id="rId8"/>
+    <hyperlink ref="B23" r:id="rId9"/>
+    <hyperlink ref="B24" r:id="rId10"/>
+    <hyperlink ref="B25" r:id="rId11"/>
+    <hyperlink ref="B26" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>

</xml_diff>

<commit_message>
Update VFD protection BOM to four-pole fused devices
Co-authored-by: XDWOLLEN <74133863+XDWOLLEN@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/pano_varyasyon_maliyet.xlsx
+++ b/pano_varyasyon_maliyet.xlsx
@@ -228,7 +228,7 @@
     <row r="7" ht="21" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Siemens SIRIUS 3RV2021-4FA10, 34–40 A motor koruma şalteri, raya montaj</t>
+          <t>Siemens SENTRON 3NP1124-1CA20, 4 kutuplu NH000 sigortalı yük ayırıcı (160 A gövde); uygun faz sigortalarıyla</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
@@ -236,8 +236,11 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C7" s="8">
+      <c r="C7" s="8" t="inlineStr">
         <v>5946.48</v>
+        <is>
+          <t>Teklif gerekli</t>
+        </is>
       </c>
       <c r="D7" s="9">
         <v>20</v>
@@ -384,7 +387,7 @@
     <row r="15" ht="21" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Teknik not: VFD çıkışında yıldız-üçgen kontaktör geçişi/zaman rölesi kullanılmaz. Motor, etiketine göre sabit yıldız veya üçgen bağlanır; hızlanma rampası sürücüden ayarlanır. Bu nedenle Pano 1 listesine Y/Δ zaman rölesi ve Y/Δ kontaktörleri eklenmemiştir.</t>
+          <t>Teknik not: VFD çıkışında yıldız-üçgen kontaktör geçişi/zaman rölesi kullanılmaz. Motor, etiketine göre sabit yıldız veya üçgen bağlanır; hızlanma rampası sürücüden ayarlanır. VFD girişinde her sürücü için 4P (3 faz + N) sigortalı ayırıcı kullanılır; N kutbunda sigorta elemanı kullanılmamalıdır. Faz sigortalarının tipi ve akımı sürücü üreticisinin koruma tablosuna göre seçilmelidir.</t>
         </is>
       </c>
     </row>
@@ -929,7 +932,7 @@
     <row r="48" ht="21" customHeight="1">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>Siemens SIRIUS 3RV2021-4FA10, 34–40 A motor koruma şalteri, raya montaj</t>
+          <t>Siemens SENTRON 3NP1124-1CA20, 4 kutuplu NH000 sigortalı yük ayırıcı (160 A gövde); uygun faz sigortalarıyla</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
@@ -940,8 +943,11 @@
       <c r="C48" s="9">
         <v>20</v>
       </c>
-      <c r="D48" s="8">
+      <c r="D48" s="8" t="inlineStr">
         <v>5946.48</v>
+        <is>
+          <t>Teklif gerekli</t>
+        </is>
       </c>
       <c r="E48" s="8">
         <f>IF(ISNUMBER(D48),C48*D48,"Teklif gerekli")</f>
@@ -1329,7 +1335,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Termik röle yerine raya montajlı Siemens 3RV2 motor koruma şalterleri listelenmiştir. Ayar aralığının motor etiket akımına uygunluğu ve sürücü öncesi koruma/koordinasyon yetkili elektrik mühendisi tarafından kontrol edilmelidir.</t>
+          <t>Pano 1 VFD giriş korumasında artık MPCB değil, 4P sigortalı ayırıcı kullanılır; nötr kutbu sigortasız olmalı, faz sigortaları sürücü talimatına göre seçilmelidir. Her 18,5 kW VFD için bir takım varsayılmıştır.</t>
         </is>
       </c>
     </row>
@@ -1438,7 +1444,7 @@
     <row r="16" ht="21" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Siemens 34–40 A MPCB</t>
+          <t>Siemens SENTRON 3NP1124-1CA20, 4P NH000 sigortalı ayırıcı</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1446,12 +1452,15 @@
           <t>Ürün sayfası</t>
         </is>
       </c>
-      <c r="C16" s="8">
+      <c r="C16" s="8" t="inlineStr">
         <v>5946.48</v>
+        <is>
+          <t>Teklif gerekli</t>
+        </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Elektrix; listelenen fiyat. Stok/fiyatı teyit edin.</t>
+          <t>Siemens ürün ailesi; 4 kutuplu NH000, 160 A gövde. Fiyat Türkiye tedarikçisi/sigorta seti için doğrulanamadı. Her VFD başına 1 takım varsayılmıştır; faz sigortaları ve nötr kutbu uygulaması Delta VFD üretici tablosu/proje hesabıyla doğrulanmalıdır.</t>
         </is>
       </c>
     </row>

</xml_diff>